<commit_message>
Use NM opportunity scoring and alerts
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3CE43F-14DE-454F-A431-1933281EBCC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C2C625-4289-473B-91F9-3767E8F51350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="11170" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="121">
   <si>
     <t>NomCarte</t>
   </si>
@@ -393,6 +393,12 @@
   </si>
   <si>
     <t>Lake of the Dead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Army of Allah (V.1) </t>
+  </si>
+  <si>
+    <t>Mono Blanc</t>
   </si>
 </sst>
 </file>
@@ -434,7 +440,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -442,17 +448,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -802,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -3565,6 +3585,23 @@
         <v>22</v>
       </c>
     </row>
+    <row r="163" spans="1:5" ht="15">
+      <c r="A163" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C163" t="s">
+        <v>6</v>
+      </c>
+      <c r="D163" t="s">
+        <v>7</v>
+      </c>
+      <c r="E163" t="s">
+        <v>120</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Sync updated collection with preserved history
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB721E3F-ED01-421D-9C58-87C921EBA182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7904D906-867E-4AB0-8F89-83BF5B303466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="19200" windowHeight="11170" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
+    <workbookView xWindow="720" yWindow="720" windowWidth="19200" windowHeight="11170" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="139">
   <si>
     <t>NomCarte</t>
   </si>
@@ -435,6 +435,24 @@
   </si>
   <si>
     <t>Land Tax</t>
+  </si>
+  <si>
+    <t>Greater Realm of Preservation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legends </t>
+  </si>
+  <si>
+    <t>Thunder Spirit</t>
+  </si>
+  <si>
+    <t>Divine Offering</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Jayemdae Tome</t>
   </si>
 </sst>
 </file>
@@ -529,13 +547,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F6F83A0D-001C-4980-961A-2565EB2F789B}" name="CollectionTable" displayName="CollectionTable" ref="A1:E125">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B3B21DC4-923F-4727-9F0C-EF5FEDA85AED}" name="CollectionTable3" displayName="CollectionTable3" ref="A1:E125">
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8E3C60EC-3A28-4C48-B9B1-1B2624CF1251}" name="NomCarte"/>
-    <tableColumn id="2" xr3:uid="{3F5E76D1-5A9D-4E9D-A780-399DCD653477}" name="Edition"/>
-    <tableColumn id="3" xr3:uid="{7274A1E9-98AA-4B2E-B956-E13C236D62E4}" name="Langue"/>
-    <tableColumn id="4" xr3:uid="{0AA597DB-18C6-4D8D-AB48-132AC534DFCB}" name="Etat"/>
-    <tableColumn id="5" xr3:uid="{9BCF75EC-B68C-49F5-BB87-21E603B55C4A}" name="Categorie"/>
+    <tableColumn id="1" xr3:uid="{1656BE50-9DE8-4279-B5FD-BB04A1DF8A62}" name="NomCarte"/>
+    <tableColumn id="2" xr3:uid="{F6028D99-F237-4CBA-A099-59A39EA0DF37}" name="Edition"/>
+    <tableColumn id="3" xr3:uid="{F65E3881-5011-4470-AF8B-04D2A7B6BD78}" name="Langue"/>
+    <tableColumn id="4" xr3:uid="{F6BC52B8-227E-45CF-AF7B-CAC3E9308A35}" name="Etat"/>
+    <tableColumn id="5" xr3:uid="{94123DB3-543C-4E9B-BF77-563B493BED4E}" name="Categorie"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -858,7 +876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E186"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -4029,6 +4047,312 @@
         <v>120</v>
       </c>
     </row>
+    <row r="187" spans="1:5" ht="15">
+      <c r="A187" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C187" t="s">
+        <v>6</v>
+      </c>
+      <c r="D187" t="s">
+        <v>10</v>
+      </c>
+      <c r="E187" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" ht="15">
+      <c r="A188" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C188" t="s">
+        <v>6</v>
+      </c>
+      <c r="D188" t="s">
+        <v>10</v>
+      </c>
+      <c r="E188" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" ht="15">
+      <c r="A189" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C189" t="s">
+        <v>36</v>
+      </c>
+      <c r="D189" t="s">
+        <v>7</v>
+      </c>
+      <c r="E189" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" ht="15">
+      <c r="A190" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C190" t="s">
+        <v>36</v>
+      </c>
+      <c r="D190" t="s">
+        <v>10</v>
+      </c>
+      <c r="E190" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" ht="15">
+      <c r="A191" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C191" t="s">
+        <v>6</v>
+      </c>
+      <c r="D191" t="s">
+        <v>7</v>
+      </c>
+      <c r="E191" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" ht="15">
+      <c r="A192" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C192" t="s">
+        <v>6</v>
+      </c>
+      <c r="D192" t="s">
+        <v>10</v>
+      </c>
+      <c r="E192" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" ht="15">
+      <c r="A193" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C193" t="s">
+        <v>6</v>
+      </c>
+      <c r="D193" t="s">
+        <v>10</v>
+      </c>
+      <c r="E193" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" ht="15">
+      <c r="A194" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C194" t="s">
+        <v>36</v>
+      </c>
+      <c r="D194" t="s">
+        <v>10</v>
+      </c>
+      <c r="E194" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" ht="15">
+      <c r="A195" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B195" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C195" t="s">
+        <v>6</v>
+      </c>
+      <c r="D195" t="s">
+        <v>10</v>
+      </c>
+      <c r="E195" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" ht="15">
+      <c r="A196" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B196" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C196" t="s">
+        <v>6</v>
+      </c>
+      <c r="D196" t="s">
+        <v>10</v>
+      </c>
+      <c r="E196" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" ht="15">
+      <c r="A197" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C197" t="s">
+        <v>6</v>
+      </c>
+      <c r="D197" t="s">
+        <v>10</v>
+      </c>
+      <c r="E197" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" ht="15">
+      <c r="A198" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B198" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C198" t="s">
+        <v>36</v>
+      </c>
+      <c r="D198" t="s">
+        <v>10</v>
+      </c>
+      <c r="E198" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" ht="15">
+      <c r="A199" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B199" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C199" t="s">
+        <v>6</v>
+      </c>
+      <c r="D199" t="s">
+        <v>10</v>
+      </c>
+      <c r="E199" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" ht="15">
+      <c r="A200" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B200" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C200" t="s">
+        <v>36</v>
+      </c>
+      <c r="D200" t="s">
+        <v>10</v>
+      </c>
+      <c r="E200" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" ht="15">
+      <c r="A201" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B201" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C201" t="s">
+        <v>6</v>
+      </c>
+      <c r="D201" t="s">
+        <v>10</v>
+      </c>
+      <c r="E201" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" ht="15">
+      <c r="A202" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B202" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C202" t="s">
+        <v>36</v>
+      </c>
+      <c r="D202" t="s">
+        <v>10</v>
+      </c>
+      <c r="E202" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" ht="15">
+      <c r="A203" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B203" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C203" t="s">
+        <v>6</v>
+      </c>
+      <c r="D203" t="s">
+        <v>49</v>
+      </c>
+      <c r="E203" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" ht="15">
+      <c r="A204" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B204" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C204" t="s">
+        <v>6</v>
+      </c>
+      <c r="D204" t="s">
+        <v>49</v>
+      </c>
+      <c r="E204" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Refresh collection and pricing simulation
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D22BF8-4827-4C90-A5DF-EEB378E7E34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E173E164-6767-4CC3-85CA-ABD02C9A13E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="1400" windowWidth="19200" windowHeight="11170" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$E$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -5589,7 +5592,7 @@
         <v>92</v>
       </c>
       <c r="C273" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="D273" s="2" t="s">
         <v>3</v>
@@ -5606,7 +5609,7 @@
         <v>92</v>
       </c>
       <c r="C274" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="D274" s="2" t="s">
         <v>3</v>
@@ -5623,7 +5626,7 @@
         <v>92</v>
       </c>
       <c r="C275" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="D275" s="2" t="s">
         <v>6</v>
@@ -5701,6 +5704,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Stabilize split JSON architecture
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6334F87-B25B-46F9-BBEF-91D332C9F297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6377F2E-44DC-43D9-9D24-D8ABA38D3963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1405" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1410" uniqueCount="164">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -528,6 +528,9 @@
   </si>
   <si>
     <t>Categorie</t>
+  </si>
+  <si>
+    <t>Rukh Egg (V.1)</t>
   </si>
 </sst>
 </file>
@@ -951,7 +954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E282"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -5737,6 +5740,23 @@
         <v>17</v>
       </c>
     </row>
+    <row r="282" spans="1:5" ht="15">
+      <c r="A282" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B282" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C282" t="s">
+        <v>2</v>
+      </c>
+      <c r="D282" t="s">
+        <v>6</v>
+      </c>
+      <c r="E282" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Sync collection from refreshed Excel file
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6377F2E-44DC-43D9-9D24-D8ABA38D3963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88960A05-8B0C-45CC-A6FE-F3C05534F554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1410" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="182">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -531,6 +531,60 @@
   </si>
   <si>
     <t>Rukh Egg (V.1)</t>
+  </si>
+  <si>
+    <t>Benalish Hero</t>
+  </si>
+  <si>
+    <t>Holy Strength</t>
+  </si>
+  <si>
+    <t>Creature Bond</t>
+  </si>
+  <si>
+    <t>Jump</t>
+  </si>
+  <si>
+    <t>Merfolk of the Pearl Trident</t>
+  </si>
+  <si>
+    <t>Terror</t>
+  </si>
+  <si>
+    <t>Weakness</t>
+  </si>
+  <si>
+    <t>Hurloon Minotaur</t>
+  </si>
+  <si>
+    <t>Giant Growth</t>
+  </si>
+  <si>
+    <t>Giant Spider</t>
+  </si>
+  <si>
+    <t>Regeneration</t>
+  </si>
+  <si>
+    <t>Scryb Sprites</t>
+  </si>
+  <si>
+    <t>Thicket Basilisk</t>
+  </si>
+  <si>
+    <t>War Mammoth</t>
+  </si>
+  <si>
+    <t>Demonic Torment</t>
+  </si>
+  <si>
+    <t>Ifh-Bíff Efreet</t>
+  </si>
+  <si>
+    <t>Wyluli Wolf (V.1)</t>
+  </si>
+  <si>
+    <t>Ivory Tower</t>
   </si>
 </sst>
 </file>
@@ -954,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E282"/>
+  <dimension ref="A1:E318"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -5757,6 +5811,618 @@
         <v>17</v>
       </c>
     </row>
+    <row r="283" spans="1:5" ht="15">
+      <c r="A283" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C283" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D283" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E283" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="284" spans="1:5" ht="15">
+      <c r="A284" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C284" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D284" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E284" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" ht="15">
+      <c r="A285" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C285" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D285" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E285" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" ht="15">
+      <c r="A286" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C286" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D286" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E286" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" ht="15">
+      <c r="A287" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C287" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D287" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E287" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="288" spans="1:5" ht="15">
+      <c r="A288" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C288" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D288" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E288" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" ht="15">
+      <c r="A289" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C289" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D289" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E289" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" ht="15">
+      <c r="A290" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C290" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D290" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E290" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" ht="15">
+      <c r="A291" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C291" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D291" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E291" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" ht="15">
+      <c r="A292" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C292" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D292" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E292" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" ht="15">
+      <c r="A293" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C293" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D293" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E293" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" ht="15">
+      <c r="A294" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C294" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D294" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E294" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" ht="15">
+      <c r="A295" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C295" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D295" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E295" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" ht="15">
+      <c r="A296" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C296" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D296" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E296" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" ht="15">
+      <c r="A297" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C297" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D297" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E297" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" ht="15">
+      <c r="A298" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B298" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C298" t="s">
+        <v>2</v>
+      </c>
+      <c r="D298" t="s">
+        <v>6</v>
+      </c>
+      <c r="E298" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" ht="15">
+      <c r="A299" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B299" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C299" t="s">
+        <v>2</v>
+      </c>
+      <c r="D299" t="s">
+        <v>6</v>
+      </c>
+      <c r="E299" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" ht="15">
+      <c r="A300" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B300" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C300" t="s">
+        <v>2</v>
+      </c>
+      <c r="D300" t="s">
+        <v>6</v>
+      </c>
+      <c r="E300" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" ht="15">
+      <c r="A301" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B301" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C301" t="s">
+        <v>2</v>
+      </c>
+      <c r="D301" t="s">
+        <v>6</v>
+      </c>
+      <c r="E301" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" ht="15">
+      <c r="A302" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B302" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C302" t="s">
+        <v>2</v>
+      </c>
+      <c r="D302" t="s">
+        <v>6</v>
+      </c>
+      <c r="E302" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="303" spans="1:5" ht="15">
+      <c r="A303" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B303" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C303" t="s">
+        <v>2</v>
+      </c>
+      <c r="D303" t="s">
+        <v>3</v>
+      </c>
+      <c r="E303" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="304" spans="1:5" ht="15">
+      <c r="A304" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B304" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C304" t="s">
+        <v>2</v>
+      </c>
+      <c r="D304" t="s">
+        <v>6</v>
+      </c>
+      <c r="E304" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="305" spans="1:5" ht="15">
+      <c r="A305" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B305" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C305" t="s">
+        <v>2</v>
+      </c>
+      <c r="D305" t="s">
+        <v>6</v>
+      </c>
+      <c r="E305" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="306" spans="1:5" ht="15">
+      <c r="A306" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B306" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C306" t="s">
+        <v>2</v>
+      </c>
+      <c r="D306" t="s">
+        <v>3</v>
+      </c>
+      <c r="E306" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="307" spans="1:5" ht="15">
+      <c r="A307" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B307" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C307" t="s">
+        <v>2</v>
+      </c>
+      <c r="D307" t="s">
+        <v>6</v>
+      </c>
+      <c r="E307" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="308" spans="1:5" ht="15">
+      <c r="A308" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B308" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C308" t="s">
+        <v>2</v>
+      </c>
+      <c r="D308" t="s">
+        <v>6</v>
+      </c>
+      <c r="E308" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="309" spans="1:5" ht="15">
+      <c r="A309" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C309" t="s">
+        <v>2</v>
+      </c>
+      <c r="D309" t="s">
+        <v>6</v>
+      </c>
+      <c r="E309" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="310" spans="1:5" ht="15">
+      <c r="A310" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C310" t="s">
+        <v>2</v>
+      </c>
+      <c r="D310" t="s">
+        <v>6</v>
+      </c>
+      <c r="E310" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="311" spans="1:5" ht="15">
+      <c r="A311" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C311" t="s">
+        <v>2</v>
+      </c>
+      <c r="D311" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E311" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="312" spans="1:5" ht="15">
+      <c r="A312" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C312" t="s">
+        <v>2</v>
+      </c>
+      <c r="D312" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E312" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="313" spans="1:5" ht="15">
+      <c r="A313" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C313" t="s">
+        <v>2</v>
+      </c>
+      <c r="D313" t="s">
+        <v>6</v>
+      </c>
+      <c r="E313" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="314" spans="1:5" ht="15">
+      <c r="A314" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C314" t="s">
+        <v>2</v>
+      </c>
+      <c r="D314" t="s">
+        <v>6</v>
+      </c>
+      <c r="E314" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="315" spans="1:5" ht="15">
+      <c r="A315" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C315" t="s">
+        <v>2</v>
+      </c>
+      <c r="D315" t="s">
+        <v>6</v>
+      </c>
+      <c r="E315" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="316" spans="1:5" ht="15">
+      <c r="A316" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C316" t="s">
+        <v>2</v>
+      </c>
+      <c r="D316" t="s">
+        <v>6</v>
+      </c>
+      <c r="E316" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="317" spans="1:5" ht="15">
+      <c r="A317" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B317" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C317" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D317" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E317" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="318" spans="1:5" ht="15">
+      <c r="A318" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B318" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C318" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D318" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E318" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Improve opportunity scoring and update collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943EA8EA-A2A2-4DD3-83E1-01993914D73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D83E23-A932-462E-BB9A-0437DBF69FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
+    <workbookView xWindow="-19125" yWindow="3075" windowWidth="19200" windowHeight="17805" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1855" uniqueCount="210">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -612,13 +612,70 @@
   </si>
   <si>
     <t>Swamp (V.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swords to Plowshares </t>
+  </si>
+  <si>
+    <t>Island Sanctuary</t>
+  </si>
+  <si>
+    <t>Wrath of God</t>
+  </si>
+  <si>
+    <t>Animate Dead</t>
+  </si>
+  <si>
+    <t>Bad Moon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lightning Bolt </t>
+  </si>
+  <si>
+    <t>Shivan Dragon</t>
+  </si>
+  <si>
+    <t>LP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Force of Nature </t>
+  </si>
+  <si>
+    <t>Howling Mine</t>
+  </si>
+  <si>
+    <t>Hell's Caretaker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concordant Crossroads </t>
+  </si>
+  <si>
+    <t>Nicol Bolas</t>
+  </si>
+  <si>
+    <t>Arena of the Ancients</t>
+  </si>
+  <si>
+    <t>Ashnod's Altar</t>
+  </si>
+  <si>
+    <t>City of Brass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sylvan Library </t>
+  </si>
+  <si>
+    <t>Fellwar Stone</t>
+  </si>
+  <si>
+    <t>Classeur2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -639,6 +696,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -653,7 +716,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -672,11 +735,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -687,6 +763,16 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1035,7 +1121,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E371"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -6620,8 +6706,740 @@
         <v>17</v>
       </c>
     </row>
+    <row r="329" spans="1:5" ht="15">
+      <c r="A329" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C329" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D329" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E329" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" ht="15">
+      <c r="A330" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C330" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D330" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E330" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" ht="15">
+      <c r="A331" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C331" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D331" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E331" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" ht="15">
+      <c r="A332" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C332" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D332" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E332" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="333" spans="1:5" ht="15">
+      <c r="A333" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C333" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D333" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E333" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="334" spans="1:5" ht="15">
+      <c r="A334" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C334" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D334" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E334" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="335" spans="1:5" ht="15">
+      <c r="A335" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C335" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D335" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E335" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="336" spans="1:5" ht="15">
+      <c r="A336" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C336" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D336" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E336" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="337" spans="1:5" ht="15">
+      <c r="A337" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C337" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D337" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E337" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="338" spans="1:5" ht="15">
+      <c r="A338" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C338" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D338" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E338" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="339" spans="1:5" ht="15">
+      <c r="A339" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C339" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D339" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E339" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="340" spans="1:5" ht="15">
+      <c r="A340" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C340" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D340" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E340" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="341" spans="1:5" ht="15">
+      <c r="A341" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C341" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D341" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="E341" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="342" spans="1:5" ht="15">
+      <c r="A342" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C342" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D342" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E342" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="343" spans="1:5" ht="15">
+      <c r="A343" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C343" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D343" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E343" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="344" spans="1:5" ht="15">
+      <c r="A344" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C344" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D344" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E344" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="345" spans="1:5" ht="15">
+      <c r="A345" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C345" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D345" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E345" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="346" spans="1:5" ht="15">
+      <c r="A346" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C346" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D346" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E346" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="347" spans="1:5" ht="15">
+      <c r="A347" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C347" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D347" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E347" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="348" spans="1:5" ht="15">
+      <c r="A348" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C348" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D348" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E348" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="349" spans="1:5" ht="15">
+      <c r="A349" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B349" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C349" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D349" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E349" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="350" spans="1:5" ht="15">
+      <c r="A350" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B350" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C350" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D350" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E350" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="351" spans="1:5" ht="15">
+      <c r="A351" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B351" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C351" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D351" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E351" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="352" spans="1:5" ht="15">
+      <c r="A352" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B352" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C352" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D352" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E352" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="353" spans="1:5" ht="15">
+      <c r="A353" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B353" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C353" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D353" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E353" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="354" spans="1:5" ht="15">
+      <c r="A354" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C354" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D354" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E354" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="355" spans="1:5" ht="15">
+      <c r="A355" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B355" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C355" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D355" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E355" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="356" spans="1:5" ht="15">
+      <c r="A356" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C356" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D356" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E356" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="357" spans="1:5" ht="15">
+      <c r="A357" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C357" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D357" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E357" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="358" spans="1:5" ht="15">
+      <c r="A358" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C358" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D358" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E358" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="359" spans="1:5" ht="15">
+      <c r="A359" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B359" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C359" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D359" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E359" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="360" spans="1:5" ht="15">
+      <c r="A360" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B360" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C360" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D360" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E360" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="361" spans="1:5" ht="15">
+      <c r="A361" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B361" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C361" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D361" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="E361" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="362" spans="1:5" ht="15">
+      <c r="A362" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B362" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C362" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D362" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E362" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="363" spans="1:5" ht="15">
+      <c r="A363" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B363" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C363" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D363" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E363" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="364" spans="1:5" ht="15">
+      <c r="A364" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B364" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C364" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D364" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E364" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="365" spans="1:5" ht="15">
+      <c r="A365" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B365" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C365" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D365" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E365" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="366" spans="1:5" ht="15">
+      <c r="A366" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B366" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C366" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D366" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E366" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="367" spans="1:5" ht="15">
+      <c r="A367" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B367" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C367" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D367" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E367" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="368" spans="1:5" ht="15">
+      <c r="A368" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B368" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C368" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D368" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E368" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="369" spans="1:5" ht="15">
+      <c r="A369" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B369" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C369" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D369" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E369" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="370" spans="1:5" ht="15">
+      <c r="A370" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B370" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C370" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D370" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E370" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="371" spans="1:5" ht="15">
+      <c r="A371" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B371" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C371" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D371" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="E371" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Add Scryfall links and update portfolio data
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D83E23-A932-462E-BB9A-0437DBF69FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{377338D8-B7E5-4B64-9171-483B7571DF82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19125" yWindow="3075" windowWidth="19200" windowHeight="17805" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
+    <workbookView xWindow="-38520" yWindow="2340" windowWidth="38640" windowHeight="21120" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1855" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1855" uniqueCount="211">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -669,6 +669,9 @@
   </si>
   <si>
     <t>Classeur2</t>
+  </si>
+  <si>
+    <t>Classeur3</t>
   </si>
 </sst>
 </file>
@@ -752,7 +755,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -764,14 +767,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3813,7 +3809,7 @@
         <v>6</v>
       </c>
       <c r="E158" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
     </row>
     <row r="159" spans="1:5" ht="15">
@@ -3830,7 +3826,7 @@
         <v>3</v>
       </c>
       <c r="E159" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
     </row>
     <row r="160" spans="1:5" ht="15">
@@ -3847,7 +3843,7 @@
         <v>3</v>
       </c>
       <c r="E160" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
     </row>
     <row r="161" spans="1:5" ht="15">
@@ -3864,7 +3860,7 @@
         <v>6</v>
       </c>
       <c r="E161" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
     </row>
     <row r="162" spans="1:5" ht="15">
@@ -3881,7 +3877,7 @@
         <v>6</v>
       </c>
       <c r="E162" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
     </row>
     <row r="163" spans="1:5" ht="15">
@@ -3898,7 +3894,7 @@
         <v>6</v>
       </c>
       <c r="E163" t="s">
-        <v>17</v>
+        <v>210</v>
       </c>
     </row>
     <row r="164" spans="1:5" ht="15">
@@ -6815,10 +6811,10 @@
       <c r="B335" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C335" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D335" s="6" t="s">
+      <c r="C335" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D335" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E335" s="2" t="s">
@@ -6832,10 +6828,10 @@
       <c r="B336" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C336" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D336" s="6" t="s">
+      <c r="C336" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D336" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E336" s="2" t="s">
@@ -6843,7 +6839,7 @@
       </c>
     </row>
     <row r="337" spans="1:5" ht="15">
-      <c r="A337" s="7" t="s">
+      <c r="A337" s="1" t="s">
         <v>195</v>
       </c>
       <c r="B337" s="1" t="s">
@@ -6860,16 +6856,16 @@
       </c>
     </row>
     <row r="338" spans="1:5" ht="15">
-      <c r="A338" s="7" t="s">
+      <c r="A338" s="1" t="s">
         <v>196</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C338" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D338" s="6" t="s">
+      <c r="C338" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D338" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E338" s="2" t="s">
@@ -6883,10 +6879,10 @@
       <c r="B339" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C339" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D339" s="6" t="s">
+      <c r="C339" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D339" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E339" s="2" t="s">
@@ -6894,16 +6890,16 @@
       </c>
     </row>
     <row r="340" spans="1:5" ht="15">
-      <c r="A340" s="7" t="s">
+      <c r="A340" s="1" t="s">
         <v>197</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C340" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D340" s="6" t="s">
+      <c r="C340" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D340" s="3" t="s">
         <v>44</v>
       </c>
       <c r="E340" s="2" t="s">
@@ -6917,10 +6913,10 @@
       <c r="B341" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C341" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D341" s="6" t="s">
+      <c r="C341" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D341" s="3" t="s">
         <v>198</v>
       </c>
       <c r="E341" s="2" t="s">
@@ -6928,16 +6924,16 @@
       </c>
     </row>
     <row r="342" spans="1:5" ht="15">
-      <c r="A342" s="7" t="s">
+      <c r="A342" s="1" t="s">
         <v>199</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C342" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D342" s="6" t="s">
+      <c r="C342" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D342" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E342" s="2" t="s">
@@ -6945,7 +6941,7 @@
       </c>
     </row>
     <row r="343" spans="1:5" ht="15">
-      <c r="A343" s="8" t="s">
+      <c r="A343" s="2" t="s">
         <v>200</v>
       </c>
       <c r="B343" s="1" t="s">
@@ -6954,7 +6950,7 @@
       <c r="C343" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D343" s="6" t="s">
+      <c r="D343" s="3" t="s">
         <v>44</v>
       </c>
       <c r="E343" s="2" t="s">
@@ -6962,16 +6958,16 @@
       </c>
     </row>
     <row r="344" spans="1:5" ht="15">
-      <c r="A344" s="7" t="s">
+      <c r="A344" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B344" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C344" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D344" s="6" t="s">
+      <c r="C344" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D344" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E344" s="2" t="s">
@@ -6979,16 +6975,16 @@
       </c>
     </row>
     <row r="345" spans="1:5" ht="15">
-      <c r="A345" s="8" t="s">
+      <c r="A345" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C345" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D345" s="6" t="s">
+      <c r="C345" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D345" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E345" s="2" t="s">
@@ -6996,7 +6992,7 @@
       </c>
     </row>
     <row r="346" spans="1:5" ht="15">
-      <c r="A346" s="7" t="s">
+      <c r="A346" s="1" t="s">
         <v>201</v>
       </c>
       <c r="B346" s="1" t="s">
@@ -7005,7 +7001,7 @@
       <c r="C346" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D346" s="6" t="s">
+      <c r="D346" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E346" s="2" t="s">
@@ -7013,7 +7009,7 @@
       </c>
     </row>
     <row r="347" spans="1:5" ht="15">
-      <c r="A347" s="8" t="s">
+      <c r="A347" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B347" s="1" t="s">
@@ -7022,7 +7018,7 @@
       <c r="C347" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D347" s="8" t="s">
+      <c r="D347" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E347" s="2" t="s">
@@ -7030,7 +7026,7 @@
       </c>
     </row>
     <row r="348" spans="1:5" ht="15">
-      <c r="A348" s="7" t="s">
+      <c r="A348" s="1" t="s">
         <v>202</v>
       </c>
       <c r="B348" s="1" t="s">
@@ -7039,7 +7035,7 @@
       <c r="C348" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D348" s="6" t="s">
+      <c r="D348" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E348" s="2" t="s">
@@ -7047,7 +7043,7 @@
       </c>
     </row>
     <row r="349" spans="1:5" ht="15">
-      <c r="A349" s="8" t="s">
+      <c r="A349" s="2" t="s">
         <v>203</v>
       </c>
       <c r="B349" s="1" t="s">
@@ -7056,7 +7052,7 @@
       <c r="C349" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D349" s="6" t="s">
+      <c r="D349" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E349" s="2" t="s">
@@ -7064,7 +7060,7 @@
       </c>
     </row>
     <row r="350" spans="1:5" ht="15">
-      <c r="A350" s="7" t="s">
+      <c r="A350" s="1" t="s">
         <v>204</v>
       </c>
       <c r="B350" s="1" t="s">
@@ -7073,7 +7069,7 @@
       <c r="C350" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D350" s="8" t="s">
+      <c r="D350" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E350" s="2" t="s">
@@ -7081,7 +7077,7 @@
       </c>
     </row>
     <row r="351" spans="1:5" ht="15">
-      <c r="A351" s="8" t="s">
+      <c r="A351" s="2" t="s">
         <v>205</v>
       </c>
       <c r="B351" s="1" t="s">
@@ -7090,7 +7086,7 @@
       <c r="C351" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D351" s="8" t="s">
+      <c r="D351" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E351" s="2" t="s">
@@ -7098,7 +7094,7 @@
       </c>
     </row>
     <row r="352" spans="1:5" ht="15">
-      <c r="A352" s="7" t="s">
+      <c r="A352" s="1" t="s">
         <v>206</v>
       </c>
       <c r="B352" s="1" t="s">
@@ -7107,7 +7103,7 @@
       <c r="C352" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D352" s="6" t="s">
+      <c r="D352" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E352" s="2" t="s">
@@ -7115,16 +7111,16 @@
       </c>
     </row>
     <row r="353" spans="1:5" ht="15">
-      <c r="A353" s="8" t="s">
+      <c r="A353" s="2" t="s">
         <v>104</v>
       </c>
       <c r="B353" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C353" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D353" s="6" t="s">
+      <c r="C353" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D353" s="3" t="s">
         <v>33</v>
       </c>
       <c r="E353" s="2" t="s">
@@ -7132,16 +7128,16 @@
       </c>
     </row>
     <row r="354" spans="1:5" ht="15">
-      <c r="A354" s="7" t="s">
+      <c r="A354" s="1" t="s">
         <v>207</v>
       </c>
       <c r="B354" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C354" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D354" s="6" t="s">
+      <c r="C354" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D354" s="3" t="s">
         <v>6</v>
       </c>
       <c r="E354" s="2" t="s">
@@ -7149,16 +7145,16 @@
       </c>
     </row>
     <row r="355" spans="1:5" ht="15">
-      <c r="A355" s="8" t="s">
+      <c r="A355" s="2" t="s">
         <v>208</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C355" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D355" s="6" t="s">
+      <c r="C355" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D355" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E355" s="2" t="s">
@@ -7166,16 +7162,16 @@
       </c>
     </row>
     <row r="356" spans="1:5" ht="15">
-      <c r="A356" s="7" t="s">
+      <c r="A356" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B356" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C356" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D356" s="6" t="s">
+      <c r="C356" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D356" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E356" s="2" t="s">
@@ -7183,7 +7179,7 @@
       </c>
     </row>
     <row r="357" spans="1:5" ht="15">
-      <c r="A357" s="8" t="s">
+      <c r="A357" s="2" t="s">
         <v>205</v>
       </c>
       <c r="B357" s="1" t="s">
@@ -7192,7 +7188,7 @@
       <c r="C357" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D357" s="8" t="s">
+      <c r="D357" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E357" s="2" t="s">
@@ -7200,7 +7196,7 @@
       </c>
     </row>
     <row r="358" spans="1:5" ht="15">
-      <c r="A358" s="8" t="s">
+      <c r="A358" s="2" t="s">
         <v>205</v>
       </c>
       <c r="B358" s="1" t="s">
@@ -7209,7 +7205,7 @@
       <c r="C358" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D358" s="8" t="s">
+      <c r="D358" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E358" s="2" t="s">
@@ -7217,7 +7213,7 @@
       </c>
     </row>
     <row r="359" spans="1:5" ht="15">
-      <c r="A359" s="8" t="s">
+      <c r="A359" s="2" t="s">
         <v>205</v>
       </c>
       <c r="B359" s="1" t="s">
@@ -7226,7 +7222,7 @@
       <c r="C359" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D359" s="8" t="s">
+      <c r="D359" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E359" s="2" t="s">
@@ -7234,7 +7230,7 @@
       </c>
     </row>
     <row r="360" spans="1:5" ht="15">
-      <c r="A360" s="7" t="s">
+      <c r="A360" s="1" t="s">
         <v>204</v>
       </c>
       <c r="B360" s="1" t="s">
@@ -7243,7 +7239,7 @@
       <c r="C360" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D360" s="8" t="s">
+      <c r="D360" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E360" s="2" t="s">
@@ -7251,16 +7247,16 @@
       </c>
     </row>
     <row r="361" spans="1:5" ht="15">
-      <c r="A361" s="7" t="s">
+      <c r="A361" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B361" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C361" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D361" s="6" t="s">
+      <c r="C361" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D361" s="3" t="s">
         <v>198</v>
       </c>
       <c r="E361" s="2" t="s">
@@ -7285,7 +7281,7 @@
       </c>
     </row>
     <row r="363" spans="1:5" ht="15">
-      <c r="A363" s="8" t="s">
+      <c r="A363" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B363" s="1" t="s">
@@ -7294,7 +7290,7 @@
       <c r="C363" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D363" s="8" t="s">
+      <c r="D363" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E363" s="2" t="s">
@@ -7302,7 +7298,7 @@
       </c>
     </row>
     <row r="364" spans="1:5" ht="15">
-      <c r="A364" s="8" t="s">
+      <c r="A364" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B364" s="1" t="s">
@@ -7311,7 +7307,7 @@
       <c r="C364" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D364" s="8" t="s">
+      <c r="D364" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E364" s="2" t="s">
@@ -7319,7 +7315,7 @@
       </c>
     </row>
     <row r="365" spans="1:5" ht="15">
-      <c r="A365" s="8" t="s">
+      <c r="A365" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B365" s="1" t="s">
@@ -7328,7 +7324,7 @@
       <c r="C365" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D365" s="8" t="s">
+      <c r="D365" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E365" s="2" t="s">
@@ -7404,16 +7400,16 @@
       </c>
     </row>
     <row r="370" spans="1:5" ht="15">
-      <c r="A370" s="7" t="s">
+      <c r="A370" s="1" t="s">
         <v>199</v>
       </c>
       <c r="B370" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C370" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D370" s="6" t="s">
+      <c r="C370" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D370" s="3" t="s">
         <v>44</v>
       </c>
       <c r="E370" s="2" t="s">
@@ -7421,16 +7417,16 @@
       </c>
     </row>
     <row r="371" spans="1:5" ht="15">
-      <c r="A371" s="8" t="s">
+      <c r="A371" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B371" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C371" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D371" s="6" t="s">
+      <c r="C371" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D371" s="3" t="s">
         <v>198</v>
       </c>
       <c r="E371" s="2" t="s">

</xml_diff>

<commit_message>
Update enrichScryfall and collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A05C080-D57B-4C6F-97AD-B9FFC7066D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447F040D-155A-438A-A8D1-EB96F873574D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2560" uniqueCount="337">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1047,6 +1047,9 @@
   </si>
   <si>
     <t>Jokulhaups</t>
+  </si>
+  <si>
+    <t>Portal Second Age</t>
   </si>
 </sst>
 </file>
@@ -1492,7 +1495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E511"/>
+  <dimension ref="A1:E512"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -10188,6 +10191,23 @@
         <v>280</v>
       </c>
     </row>
+    <row r="512" spans="1:5" ht="15">
+      <c r="A512" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B512" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="C512" t="s">
+        <v>31</v>
+      </c>
+      <c r="D512" t="s">
+        <v>6</v>
+      </c>
+      <c r="E512" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Update collection and portfolio data
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447F040D-155A-438A-A8D1-EB96F873574D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3355A800-5091-44AC-A0A0-BEF829C8A946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2560" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="371">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1050,6 +1050,108 @@
   </si>
   <si>
     <t>Portal Second Age</t>
+  </si>
+  <si>
+    <t>Energy Storm</t>
+  </si>
+  <si>
+    <t>Ice Age</t>
+  </si>
+  <si>
+    <t>Enduring Renewal</t>
+  </si>
+  <si>
+    <t>Polar Kraken</t>
+  </si>
+  <si>
+    <t>Dance of the Dead</t>
+  </si>
+  <si>
+    <t>Burnt Offering</t>
+  </si>
+  <si>
+    <t>Songs of the Damned</t>
+  </si>
+  <si>
+    <t>Pyroblast </t>
+  </si>
+  <si>
+    <t>Anarchy </t>
+  </si>
+  <si>
+    <t>Jokulhaups </t>
+  </si>
+  <si>
+    <t>Pyroclasm </t>
+  </si>
+  <si>
+    <t>Balduvian Hydra</t>
+  </si>
+  <si>
+    <t>Thermokarst</t>
+  </si>
+  <si>
+    <t>Nature's Lore</t>
+  </si>
+  <si>
+    <t>Fyndhorn Elves</t>
+  </si>
+  <si>
+    <t>Lhurgoyf</t>
+  </si>
+  <si>
+    <t>Jeweled Amulet</t>
+  </si>
+  <si>
+    <t>Fire Covenant</t>
+  </si>
+  <si>
+    <t>Snow-Covered Plains</t>
+  </si>
+  <si>
+    <t>Snow-Covered Island</t>
+  </si>
+  <si>
+    <t>Snow-Covered Swamp</t>
+  </si>
+  <si>
+    <t>Snow-Covered Forest</t>
+  </si>
+  <si>
+    <t>Adarkar Wastes</t>
+  </si>
+  <si>
+    <t>Glacial Chasm</t>
+  </si>
+  <si>
+    <t>Karplusan Forest</t>
+  </si>
+  <si>
+    <t>Brushland </t>
+  </si>
+  <si>
+    <t>Soraya the Falconer</t>
+  </si>
+  <si>
+    <t>Homelands </t>
+  </si>
+  <si>
+    <t>Serra Aviary</t>
+  </si>
+  <si>
+    <t>Baron Sengir</t>
+  </si>
+  <si>
+    <t>Koskun Falls</t>
+  </si>
+  <si>
+    <t>Veldrane of Sengir </t>
+  </si>
+  <si>
+    <t>An-Zerrin Ruins</t>
+  </si>
+  <si>
+    <t>Didgeridoo </t>
   </si>
 </sst>
 </file>
@@ -1495,7 +1597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E512"/>
+  <dimension ref="A1:E546"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -10208,6 +10310,584 @@
         <v>280</v>
       </c>
     </row>
+    <row r="513" spans="1:5" ht="15">
+      <c r="A513" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B513" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C513" t="s">
+        <v>31</v>
+      </c>
+      <c r="D513" t="s">
+        <v>6</v>
+      </c>
+      <c r="E513" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="514" spans="1:5" ht="15">
+      <c r="A514" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B514" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C514" t="s">
+        <v>31</v>
+      </c>
+      <c r="D514" t="s">
+        <v>6</v>
+      </c>
+      <c r="E514" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="515" spans="1:5" ht="15">
+      <c r="A515" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B515" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C515" t="s">
+        <v>31</v>
+      </c>
+      <c r="D515" t="s">
+        <v>6</v>
+      </c>
+      <c r="E515" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="516" spans="1:5" ht="15">
+      <c r="A516" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B516" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C516" t="s">
+        <v>2</v>
+      </c>
+      <c r="D516" t="s">
+        <v>33</v>
+      </c>
+      <c r="E516" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="517" spans="1:5" ht="15">
+      <c r="A517" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B517" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C517" t="s">
+        <v>31</v>
+      </c>
+      <c r="D517" t="s">
+        <v>3</v>
+      </c>
+      <c r="E517" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="518" spans="1:5" ht="15">
+      <c r="A518" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B518" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C518" t="s">
+        <v>2</v>
+      </c>
+      <c r="D518" t="s">
+        <v>44</v>
+      </c>
+      <c r="E518" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="519" spans="1:5" ht="15">
+      <c r="A519" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B519" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C519" t="s">
+        <v>2</v>
+      </c>
+      <c r="D519" t="s">
+        <v>44</v>
+      </c>
+      <c r="E519" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="520" spans="1:5" ht="15">
+      <c r="A520" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B520" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C520" t="s">
+        <v>2</v>
+      </c>
+      <c r="D520" t="s">
+        <v>6</v>
+      </c>
+      <c r="E520" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="521" spans="1:5" ht="15">
+      <c r="A521" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="B521" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C521" t="s">
+        <v>31</v>
+      </c>
+      <c r="D521" t="s">
+        <v>198</v>
+      </c>
+      <c r="E521" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="522" spans="1:5" ht="15">
+      <c r="A522" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B522" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C522" t="s">
+        <v>2</v>
+      </c>
+      <c r="D522" t="s">
+        <v>44</v>
+      </c>
+      <c r="E522" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="523" spans="1:5" ht="15">
+      <c r="A523" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B523" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C523" t="s">
+        <v>31</v>
+      </c>
+      <c r="D523" t="s">
+        <v>6</v>
+      </c>
+      <c r="E523" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="524" spans="1:5" ht="15">
+      <c r="A524" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="B524" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C524" t="s">
+        <v>31</v>
+      </c>
+      <c r="D524" t="s">
+        <v>3</v>
+      </c>
+      <c r="E524" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="525" spans="1:5" ht="15">
+      <c r="A525" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="B525" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C525" t="s">
+        <v>31</v>
+      </c>
+      <c r="D525" t="s">
+        <v>44</v>
+      </c>
+      <c r="E525" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="526" spans="1:5" ht="15">
+      <c r="A526" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B526" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C526" t="s">
+        <v>31</v>
+      </c>
+      <c r="D526" t="s">
+        <v>44</v>
+      </c>
+      <c r="E526" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="527" spans="1:5" ht="15">
+      <c r="A527" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="B527" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C527" t="s">
+        <v>2</v>
+      </c>
+      <c r="D527" t="s">
+        <v>6</v>
+      </c>
+      <c r="E527" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="528" spans="1:5" ht="15">
+      <c r="A528" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="B528" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C528" t="s">
+        <v>2</v>
+      </c>
+      <c r="D528" t="s">
+        <v>198</v>
+      </c>
+      <c r="E528" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="529" spans="1:5" ht="15">
+      <c r="A529" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B529" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C529" t="s">
+        <v>2</v>
+      </c>
+      <c r="D529" t="s">
+        <v>33</v>
+      </c>
+      <c r="E529" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="530" spans="1:5" ht="15">
+      <c r="A530" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="B530" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C530" t="s">
+        <v>2</v>
+      </c>
+      <c r="D530" t="s">
+        <v>44</v>
+      </c>
+      <c r="E530" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="531" spans="1:5" ht="15">
+      <c r="A531" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B531" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C531" t="s">
+        <v>31</v>
+      </c>
+      <c r="D531" t="s">
+        <v>44</v>
+      </c>
+      <c r="E531" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="532" spans="1:5" ht="15">
+      <c r="A532" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B532" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C532" t="s">
+        <v>31</v>
+      </c>
+      <c r="D532" t="s">
+        <v>44</v>
+      </c>
+      <c r="E532" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="533" spans="1:5" ht="15">
+      <c r="A533" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B533" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C533" t="s">
+        <v>2</v>
+      </c>
+      <c r="D533" t="s">
+        <v>6</v>
+      </c>
+      <c r="E533" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="534" spans="1:5" ht="15">
+      <c r="A534" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="B534" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C534" t="s">
+        <v>2</v>
+      </c>
+      <c r="D534" t="s">
+        <v>6</v>
+      </c>
+      <c r="E534" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="535" spans="1:5" ht="15">
+      <c r="A535" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B535" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C535" t="s">
+        <v>2</v>
+      </c>
+      <c r="D535" t="s">
+        <v>6</v>
+      </c>
+      <c r="E535" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="536" spans="1:5" ht="15">
+      <c r="A536" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B536" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C536" t="s">
+        <v>2</v>
+      </c>
+      <c r="D536" t="s">
+        <v>6</v>
+      </c>
+      <c r="E536" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="537" spans="1:5" ht="15">
+      <c r="A537" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B537" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C537" t="s">
+        <v>2</v>
+      </c>
+      <c r="D537" t="s">
+        <v>6</v>
+      </c>
+      <c r="E537" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="538" spans="1:5" ht="15">
+      <c r="A538" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B538" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C538" t="s">
+        <v>31</v>
+      </c>
+      <c r="D538" t="s">
+        <v>6</v>
+      </c>
+      <c r="E538" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="539" spans="1:5" ht="15">
+      <c r="A539" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="B539" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C539" t="s">
+        <v>31</v>
+      </c>
+      <c r="D539" t="s">
+        <v>6</v>
+      </c>
+      <c r="E539" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="540" spans="1:5" ht="15">
+      <c r="A540" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B540" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C540" t="s">
+        <v>31</v>
+      </c>
+      <c r="D540" t="s">
+        <v>3</v>
+      </c>
+      <c r="E540" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="541" spans="1:5" ht="15">
+      <c r="A541" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B541" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C541" t="s">
+        <v>31</v>
+      </c>
+      <c r="D541" t="s">
+        <v>44</v>
+      </c>
+      <c r="E541" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="542" spans="1:5" ht="15">
+      <c r="A542" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B542" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C542" t="s">
+        <v>31</v>
+      </c>
+      <c r="D542" t="s">
+        <v>3</v>
+      </c>
+      <c r="E542" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="543" spans="1:5" ht="15">
+      <c r="A543" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B543" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C543" t="s">
+        <v>31</v>
+      </c>
+      <c r="D543" t="s">
+        <v>6</v>
+      </c>
+      <c r="E543" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="544" spans="1:5" ht="15">
+      <c r="A544" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="B544" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C544" t="s">
+        <v>31</v>
+      </c>
+      <c r="D544" t="s">
+        <v>44</v>
+      </c>
+      <c r="E544" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="545" spans="1:5" ht="15">
+      <c r="A545" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B545" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C545" t="s">
+        <v>2</v>
+      </c>
+      <c r="D545" t="s">
+        <v>41</v>
+      </c>
+      <c r="E545" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="546" spans="1:5" ht="15">
+      <c r="A546" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B546" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C546" t="s">
+        <v>2</v>
+      </c>
+      <c r="D546" t="s">
+        <v>33</v>
+      </c>
+      <c r="E546" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Fix portfolio export and update collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3355A800-5091-44AC-A0A0-BEF829C8A946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670CF89D-1473-4010-AF91-9DEA7D390E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2935" uniqueCount="377">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1152,6 +1152,24 @@
   </si>
   <si>
     <t>Didgeridoo </t>
+  </si>
+  <si>
+    <t>Blanc Vert</t>
+  </si>
+  <si>
+    <t>Savannah</t>
+  </si>
+  <si>
+    <t>Foreign White Border</t>
+  </si>
+  <si>
+    <t>Spirit Link</t>
+  </si>
+  <si>
+    <t>Regrowth</t>
+  </si>
+  <si>
+    <t>Tsunami</t>
   </si>
 </sst>
 </file>
@@ -1186,7 +1204,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1198,8 +1216,14 @@
         <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1231,11 +1255,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1248,6 +1285,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1597,7 +1646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E546"/>
+  <dimension ref="A1:E587"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -10888,6 +10937,703 @@
         <v>210</v>
       </c>
     </row>
+    <row r="547" spans="1:5">
+      <c r="A547" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B547" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C547" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D547" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E547" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="548" spans="1:5" ht="15">
+      <c r="A548" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B548" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C548" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D548" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E548" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="549" spans="1:5" ht="15">
+      <c r="A549" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B549" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C549" t="s">
+        <v>2</v>
+      </c>
+      <c r="D549" t="s">
+        <v>6</v>
+      </c>
+      <c r="E549" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="550" spans="1:5" ht="15">
+      <c r="A550" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B550" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C550" t="s">
+        <v>2</v>
+      </c>
+      <c r="D550" t="s">
+        <v>44</v>
+      </c>
+      <c r="E550" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="551" spans="1:5">
+      <c r="A551" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B551" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="C551" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D551" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E551" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="552" spans="1:5" ht="15">
+      <c r="A552" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B552" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C552" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D552" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E552" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="553" spans="1:5" ht="15">
+      <c r="A553" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B553" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="C553" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D553" t="s">
+        <v>6</v>
+      </c>
+      <c r="E553" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="554" spans="1:5" ht="15">
+      <c r="A554" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B554" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C554" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D554" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E554" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="555" spans="1:5">
+      <c r="A555" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B555" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C555" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D555" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E555" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="556" spans="1:5">
+      <c r="A556" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B556" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C556" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D556" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E556" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="557" spans="1:5" ht="15">
+      <c r="A557" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B557" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C557" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D557" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E557" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="558" spans="1:5" ht="15">
+      <c r="A558" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B558" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C558" t="s">
+        <v>2</v>
+      </c>
+      <c r="D558" t="s">
+        <v>6</v>
+      </c>
+      <c r="E558" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="559" spans="1:5" ht="15">
+      <c r="A559" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B559" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C559" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D559" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E559" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="560" spans="1:5" ht="15">
+      <c r="A560" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B560" t="s">
+        <v>129</v>
+      </c>
+      <c r="C560" t="s">
+        <v>2</v>
+      </c>
+      <c r="D560" t="s">
+        <v>6</v>
+      </c>
+      <c r="E560" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="561" spans="1:5">
+      <c r="A561" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B561" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C561" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D561" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E561" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="562" spans="1:5" ht="15">
+      <c r="A562" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B562" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C562" t="s">
+        <v>2</v>
+      </c>
+      <c r="D562" t="s">
+        <v>3</v>
+      </c>
+      <c r="E562" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="563" spans="1:5" ht="15">
+      <c r="A563" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B563" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C563" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D563" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E563" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="564" spans="1:5" ht="15">
+      <c r="A564" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B564" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C564" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D564" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E564" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="565" spans="1:5" ht="15">
+      <c r="A565" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B565" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C565" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D565" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E565" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="566" spans="1:5" ht="15">
+      <c r="A566" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B566" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C566" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D566" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E566" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="567" spans="1:5" ht="15">
+      <c r="A567" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B567" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C567" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D567" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E567" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="568" spans="1:5">
+      <c r="A568" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B568" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C568" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D568" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E568" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="569" spans="1:5" ht="15">
+      <c r="A569" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B569" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C569" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D569" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E569" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="570" spans="1:5">
+      <c r="A570" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B570" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C570" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D570" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E570" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="571" spans="1:5" ht="15">
+      <c r="A571" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B571" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C571" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D571" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E571" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="572" spans="1:5">
+      <c r="A572" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B572" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C572" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D572" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E572" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="573" spans="1:5">
+      <c r="A573" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B573" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C573" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D573" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E573" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="574" spans="1:5" ht="15">
+      <c r="A574" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B574" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C574" t="s">
+        <v>2</v>
+      </c>
+      <c r="D574" t="s">
+        <v>6</v>
+      </c>
+      <c r="E574" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="575" spans="1:5" ht="15">
+      <c r="A575" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B575" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="C575" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D575" t="s">
+        <v>6</v>
+      </c>
+      <c r="E575" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="576" spans="1:5">
+      <c r="A576" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B576" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C576" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D576" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E576" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="577" spans="1:5">
+      <c r="A577" t="s">
+        <v>76</v>
+      </c>
+      <c r="B577" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C577" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D577" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E577" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="578" spans="1:5">
+      <c r="A578" t="s">
+        <v>132</v>
+      </c>
+      <c r="B578" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C578" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D578" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E578" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="579" spans="1:5" ht="15">
+      <c r="A579" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B579" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C579" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D579" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E579" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="580" spans="1:5" ht="15">
+      <c r="A580" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B580" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C580" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D580" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E580" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="581" spans="1:5">
+      <c r="A581" t="s">
+        <v>375</v>
+      </c>
+      <c r="B581" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C581" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D581" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E581" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="582" spans="1:5">
+      <c r="A582" t="s">
+        <v>376</v>
+      </c>
+      <c r="B582" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C582" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D582" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E582" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="583" spans="1:5">
+      <c r="A583" t="s">
+        <v>127</v>
+      </c>
+      <c r="B583" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C583" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D583" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E583" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="584" spans="1:5">
+      <c r="A584" t="s">
+        <v>127</v>
+      </c>
+      <c r="B584" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C584" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D584" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E584" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="585" spans="1:5" ht="15">
+      <c r="A585" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B585" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C585" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D585" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E585" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="586" spans="1:5" ht="15">
+      <c r="A586" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B586" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C586" t="s">
+        <v>2</v>
+      </c>
+      <c r="D586" t="s">
+        <v>198</v>
+      </c>
+      <c r="E586" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="587" spans="1:5">
+      <c r="A587" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B587" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="C587" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D587" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E587" s="7" t="s">
+        <v>371</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Group collection cards by card and variant
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6D9989-8145-45F4-8EC5-4DAEA95700EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AC8B20-106C-436C-93EC-BE4E090E8CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3220" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3250" uniqueCount="425">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1302,6 +1302,18 @@
   </si>
   <si>
     <t>Wandering Mage</t>
+  </si>
+  <si>
+    <t>Balduvian Trading Post</t>
+  </si>
+  <si>
+    <t>Sheltered Valley</t>
+  </si>
+  <si>
+    <t>German</t>
+  </si>
+  <si>
+    <t>Control Magic</t>
   </si>
 </sst>
 </file>
@@ -1781,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E644"/>
+  <dimension ref="A1:E650"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -12738,6 +12750,108 @@
         <v>367</v>
       </c>
     </row>
+    <row r="645" spans="1:5" ht="15">
+      <c r="A645" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B645" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C645" t="s">
+        <v>29</v>
+      </c>
+      <c r="D645" t="s">
+        <v>3</v>
+      </c>
+      <c r="E645" s="2" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="646" spans="1:5" ht="15">
+      <c r="A646" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="B646" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C646" t="s">
+        <v>29</v>
+      </c>
+      <c r="D646" t="s">
+        <v>6</v>
+      </c>
+      <c r="E646" s="2" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="647" spans="1:5" ht="15">
+      <c r="A647" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B647" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C647" t="s">
+        <v>29</v>
+      </c>
+      <c r="D647" t="s">
+        <v>6</v>
+      </c>
+      <c r="E647" s="2" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="648" spans="1:5" ht="15">
+      <c r="A648" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B648" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C648" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D648" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E648" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="649" spans="1:5" ht="15">
+      <c r="A649" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B649" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C649" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D649" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E649" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="650" spans="1:5" ht="15">
+      <c r="A650" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B650" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C650" t="s">
+        <v>29</v>
+      </c>
+      <c r="D650" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E650" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Group card artwork variants in collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AC8B20-106C-436C-93EC-BE4E090E8CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E201C4-49F0-42CA-86B8-DE8FD94971C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3250" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3255" uniqueCount="425">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1793,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E650"/>
+  <dimension ref="A1:E651"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -12852,6 +12852,23 @@
         <v>366</v>
       </c>
     </row>
+    <row r="651" spans="1:5" ht="15">
+      <c r="A651" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B651" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C651" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D651" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E651" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Show collection categories under card names
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E201C4-49F0-42CA-86B8-DE8FD94971C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED90378-5D55-4B8A-A56D-E211478FBC52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3255" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3280" uniqueCount="428">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1314,6 +1314,15 @@
   </si>
   <si>
     <t>Control Magic</t>
+  </si>
+  <si>
+    <t>Nightmare </t>
+  </si>
+  <si>
+    <t>Mana Flare</t>
+  </si>
+  <si>
+    <t>Instill Energy</t>
   </si>
 </sst>
 </file>
@@ -1416,7 +1425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1444,6 +1453,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1793,7 +1808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E651"/>
+  <dimension ref="A1:E656"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -12869,6 +12884,91 @@
         <v>366</v>
       </c>
     </row>
+    <row r="652" spans="1:5" ht="15">
+      <c r="A652" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="B652" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C652" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D652" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E652" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="653" spans="1:5" ht="15">
+      <c r="A653" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B653" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C653" t="s">
+        <v>29</v>
+      </c>
+      <c r="D653" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E653" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="654" spans="1:5" ht="15">
+      <c r="A654" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="B654" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C654" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D654" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E654" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="655" spans="1:5" ht="15">
+      <c r="A655" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B655" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C655" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D655" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E655" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="656" spans="1:5" ht="15">
+      <c r="A656" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B656" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C656" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D656" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E656" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Add collection edition filter and sort variants by price
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6214CFB-E563-423A-8FC2-139FD5978ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADD0415-8C94-437E-BAAA-1A371B40EDB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4030" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4230" uniqueCount="508">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1485,6 +1485,84 @@
   </si>
   <si>
     <t>Repentant Blacksmith</t>
+  </si>
+  <si>
+    <t>Spectral Guardian</t>
+  </si>
+  <si>
+    <t>Dark Ritual </t>
+  </si>
+  <si>
+    <t>Dwarven Miner</t>
+  </si>
+  <si>
+    <t>Telim'Tor</t>
+  </si>
+  <si>
+    <t>Volcanic Dragon</t>
+  </si>
+  <si>
+    <t>Uktabi Wildcats</t>
+  </si>
+  <si>
+    <t>Wall of Roots</t>
+  </si>
+  <si>
+    <t>Benthic Djinn</t>
+  </si>
+  <si>
+    <t>Energy Bolt</t>
+  </si>
+  <si>
+    <t>Rocky Tar Pit</t>
+  </si>
+  <si>
+    <t>Mountain Valley</t>
+  </si>
+  <si>
+    <t>Eye of Singularity</t>
+  </si>
+  <si>
+    <t>Zhalfirin Crusader</t>
+  </si>
+  <si>
+    <t>Flooded Shoreline</t>
+  </si>
+  <si>
+    <t>Impulse</t>
+  </si>
+  <si>
+    <t>Prosperity </t>
+  </si>
+  <si>
+    <t>Rainbow Efreet</t>
+  </si>
+  <si>
+    <t>Vision Charm</t>
+  </si>
+  <si>
+    <t>Crypt Rats</t>
+  </si>
+  <si>
+    <t>Bogardan Phoenix</t>
+  </si>
+  <si>
+    <t>Fireblast</t>
+  </si>
+  <si>
+    <t>Ogre Enforcer</t>
+  </si>
+  <si>
+    <t>Katabatic Winds</t>
+  </si>
+  <si>
+    <t>Quirion Druid</t>
+  </si>
+  <si>
+    <t>Uktabi Orangutan</t>
+  </si>
+  <si>
+    <t>Snake Basket</t>
   </si>
 </sst>
 </file>
@@ -1603,7 +1681,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1634,10 +1712,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1987,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E806"/>
+  <dimension ref="A1:E846"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -15419,7 +15500,7 @@
       <c r="C790" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D790" s="13" t="s">
+      <c r="D790" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E790" s="12" t="s">
@@ -15436,7 +15517,7 @@
       <c r="C791" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D791" s="13" t="s">
+      <c r="D791" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E791" s="12" t="s">
@@ -15453,7 +15534,7 @@
       <c r="C792" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D792" s="13" t="s">
+      <c r="D792" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E792" s="12" t="s">
@@ -15470,7 +15551,7 @@
       <c r="C793" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D793" s="13" t="s">
+      <c r="D793" s="2" t="s">
         <v>42</v>
       </c>
       <c r="E793" s="12" t="s">
@@ -15487,7 +15568,7 @@
       <c r="C794" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D794" s="13" t="s">
+      <c r="D794" s="2" t="s">
         <v>192</v>
       </c>
       <c r="E794" s="12" t="s">
@@ -15504,7 +15585,7 @@
       <c r="C795" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D795" s="13" t="s">
+      <c r="D795" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E795" s="12" t="s">
@@ -15521,7 +15602,7 @@
       <c r="C796" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D796" s="13" t="s">
+      <c r="D796" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E796" s="12" t="s">
@@ -15538,7 +15619,7 @@
       <c r="C797" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D797" s="13" t="s">
+      <c r="D797" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E797" s="12" t="s">
@@ -15555,7 +15636,7 @@
       <c r="C798" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D798" s="13" t="s">
+      <c r="D798" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E798" s="12" t="s">
@@ -15572,7 +15653,7 @@
       <c r="C799" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D799" s="13" t="s">
+      <c r="D799" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E799" s="12" t="s">
@@ -15589,7 +15670,7 @@
       <c r="C800" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D800" s="13" t="s">
+      <c r="D800" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E800" s="12" t="s">
@@ -15640,7 +15721,7 @@
       <c r="C803" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D803" s="13" t="s">
+      <c r="D803" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E803" s="12" t="s">
@@ -15657,7 +15738,7 @@
       <c r="C804" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D804" s="13" t="s">
+      <c r="D804" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E804" s="12" t="s">
@@ -15674,7 +15755,7 @@
       <c r="C805" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D805" s="13" t="s">
+      <c r="D805" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E805" s="12" t="s">
@@ -15696,6 +15777,686 @@
       </c>
       <c r="E806" s="12" t="s">
         <v>374</v>
+      </c>
+    </row>
+    <row r="807" spans="1:5" ht="15">
+      <c r="A807" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B807" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C807" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D807" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E807" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="808" spans="1:5" ht="15">
+      <c r="A808" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B808" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C808" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D808" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E808" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="809" spans="1:5" ht="15">
+      <c r="A809" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B809" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C809" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D809" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E809" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="810" spans="1:5" ht="15">
+      <c r="A810" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B810" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C810" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D810" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E810" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="811" spans="1:5" ht="15">
+      <c r="A811" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B811" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C811" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D811" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E811" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="812" spans="1:5" ht="15">
+      <c r="A812" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B812" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C812" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D812" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E812" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="813" spans="1:5" ht="15">
+      <c r="A813" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B813" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C813" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D813" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E813" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="814" spans="1:5" ht="15">
+      <c r="A814" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B814" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C814" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D814" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E814" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="815" spans="1:5" ht="15">
+      <c r="A815" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B815" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C815" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D815" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E815" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="816" spans="1:5" ht="15">
+      <c r="A816" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B816" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C816" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D816" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E816" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="817" spans="1:5" ht="15">
+      <c r="A817" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B817" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C817" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D817" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E817" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="818" spans="1:5" ht="15">
+      <c r="A818" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B818" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C818" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D818" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E818" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="819" spans="1:5" ht="15">
+      <c r="A819" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B819" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C819" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D819" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E819" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="820" spans="1:5" ht="15">
+      <c r="A820" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B820" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C820" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D820" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E820" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="821" spans="1:5" ht="15">
+      <c r="A821" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="B821" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C821" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D821" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E821" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="822" spans="1:5" ht="15">
+      <c r="A822" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B822" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C822" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D822" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E822" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="823" spans="1:5" ht="15">
+      <c r="A823" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="B823" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C823" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D823" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E823" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="824" spans="1:5" ht="15">
+      <c r="A824" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B824" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C824" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D824" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E824" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="825" spans="1:5" ht="15">
+      <c r="A825" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="B825" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C825" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D825" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E825" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="826" spans="1:5" ht="15">
+      <c r="A826" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B826" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C826" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D826" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E826" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="827" spans="1:5" ht="15">
+      <c r="A827" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B827" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C827" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D827" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E827" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="828" spans="1:5" ht="15">
+      <c r="A828" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B828" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C828" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D828" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E828" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="829" spans="1:5" ht="15">
+      <c r="A829" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B829" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C829" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D829" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E829" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="830" spans="1:5" ht="15">
+      <c r="A830" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="B830" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C830" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D830" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E830" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="831" spans="1:5" ht="15">
+      <c r="A831" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="B831" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C831" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D831" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E831" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="832" spans="1:5" ht="15">
+      <c r="A832" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="B832" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C832" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D832" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E832" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="833" spans="1:5" ht="15">
+      <c r="A833" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="B833" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C833" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D833" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E833" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="834" spans="1:5" ht="15">
+      <c r="A834" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="B834" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C834" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D834" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E834" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="835" spans="1:5" ht="15">
+      <c r="A835" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="B835" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C835" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D835" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E835" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="836" spans="1:5" ht="15">
+      <c r="A836" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="B836" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C836" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D836" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E836" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="837" spans="1:5" ht="15">
+      <c r="A837" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="B837" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C837" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D837" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E837" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="838" spans="1:5" ht="15">
+      <c r="A838" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B838" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C838" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D838" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E838" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="839" spans="1:5" ht="15">
+      <c r="A839" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B839" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C839" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D839" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E839" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="840" spans="1:5" ht="15">
+      <c r="A840" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B840" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C840" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D840" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E840" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="841" spans="1:5" ht="15">
+      <c r="A841" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="B841" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C841" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D841" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E841" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="842" spans="1:5" ht="15">
+      <c r="A842" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="B842" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C842" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D842" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E842" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="843" spans="1:5" ht="15">
+      <c r="A843" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="B843" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C843" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D843" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E843" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="844" spans="1:5" ht="15">
+      <c r="A844" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B844" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C844" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D844" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E844" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="845" spans="1:5" ht="15">
+      <c r="A845" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="B845" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C845" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D845" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E845" s="13" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="846" spans="1:5" ht="15">
+      <c r="A846" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="B846" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C846" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D846" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="E846" s="13" t="s">
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Radar filter and column layout
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FFD26A-5E2F-4ADB-BA14-EAC59D09C293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940515BC-B5EE-4747-8828-E52F6ACF1642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4380" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4385" uniqueCount="528">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -2122,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E876"/>
+  <dimension ref="A1:E877"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -17023,6 +17023,23 @@
         <v>368</v>
       </c>
     </row>
+    <row r="877" spans="1:5" ht="15">
+      <c r="A877" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B877" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C877" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D877" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E877" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Update collection and fix Radar email alerts
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940515BC-B5EE-4747-8828-E52F6ACF1642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B261438-5604-44A6-84E2-9DF90693E1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4385" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5295" uniqueCount="584">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1623,13 +1623,181 @@
   </si>
   <si>
     <t>Time Warp</t>
+  </si>
+  <si>
+    <t>Artifact Ward</t>
+  </si>
+  <si>
+    <t>Reconstruction</t>
+  </si>
+  <si>
+    <t>Artifact Possession</t>
+  </si>
+  <si>
+    <t>Orcish Mechanics</t>
+  </si>
+  <si>
+    <t>Argothian Treefolk</t>
+  </si>
+  <si>
+    <t>Amulet of Kroog</t>
+  </si>
+  <si>
+    <t>Battering Ram</t>
+  </si>
+  <si>
+    <t>Clay Statue</t>
+  </si>
+  <si>
+    <t>Dragon Engine</t>
+  </si>
+  <si>
+    <t>Tablet of Epityr</t>
+  </si>
+  <si>
+    <t>Urza's Chalice</t>
+  </si>
+  <si>
+    <t>Yotian Soldier</t>
+  </si>
+  <si>
+    <t>Pirate Ship</t>
+  </si>
+  <si>
+    <t>Kird Ape</t>
+  </si>
+  <si>
+    <t>Crumble</t>
+  </si>
+  <si>
+    <t>Island (V.3)</t>
+  </si>
+  <si>
+    <t>Plains (V.3)</t>
+  </si>
+  <si>
+    <t>Swamp (V.2)</t>
+  </si>
+  <si>
+    <t>Mountain (V.3)</t>
+  </si>
+  <si>
+    <t>Mountain (V.2)</t>
+  </si>
+  <si>
+    <t>Power Surge</t>
+  </si>
+  <si>
+    <t>Titania's Song</t>
+  </si>
+  <si>
+    <t>Millstone </t>
+  </si>
+  <si>
+    <t>Disrupting Scepter</t>
+  </si>
+  <si>
+    <t>Amrou Kithkin</t>
+  </si>
+  <si>
+    <t>Legends </t>
+  </si>
+  <si>
+    <t>Clergy of the Holy Nimbus</t>
+  </si>
+  <si>
+    <t>Anti-Magic Aura</t>
+  </si>
+  <si>
+    <t>Flash Counter</t>
+  </si>
+  <si>
+    <t>Gaseous Form</t>
+  </si>
+  <si>
+    <t>Glyph of Delusion</t>
+  </si>
+  <si>
+    <t>Remove Soul</t>
+  </si>
+  <si>
+    <t>Wall of Vapor</t>
+  </si>
+  <si>
+    <t>Transmutation</t>
+  </si>
+  <si>
+    <t>Active Volcano</t>
+  </si>
+  <si>
+    <t>Blazing Effigy</t>
+  </si>
+  <si>
+    <t>Pyrotechnics </t>
+  </si>
+  <si>
+    <t>Raging Bull</t>
+  </si>
+  <si>
+    <t>The Brute</t>
+  </si>
+  <si>
+    <t>Wall of Earth</t>
+  </si>
+  <si>
+    <t>Aisling Leprechaun</t>
+  </si>
+  <si>
+    <t>Fire Sprites</t>
+  </si>
+  <si>
+    <t>Subdue</t>
+  </si>
+  <si>
+    <t>Rust</t>
+  </si>
+  <si>
+    <t>Fire and Brimstone</t>
+  </si>
+  <si>
+    <t>Electric Eel</t>
+  </si>
+  <si>
+    <t>Ghost Ship</t>
+  </si>
+  <si>
+    <t>Banshee</t>
+  </si>
+  <si>
+    <t>The Fallen</t>
+  </si>
+  <si>
+    <t>Goblin Caves</t>
+  </si>
+  <si>
+    <t>Orc General</t>
+  </si>
+  <si>
+    <t>People of the Woods</t>
+  </si>
+  <si>
+    <t>Scarwood Hag</t>
+  </si>
+  <si>
+    <t>Whippoorwill</t>
+  </si>
+  <si>
+    <t>Standing Stones</t>
+  </si>
+  <si>
+    <t>Evil Presence </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1663,6 +1831,13 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="26.85"/>
+      <color rgb="FFE4E6EB"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1683,7 +1858,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1737,11 +1912,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1773,6 +1957,33 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2122,7 +2333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E877"/>
+  <dimension ref="A1:E1059"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -2754,7 +2965,7 @@
         <v>29</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>365</v>
@@ -15744,8 +15955,8 @@
       <c r="D801" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E801" s="7" t="s">
-        <v>375</v>
+      <c r="E801" s="12" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="802" spans="1:5" ht="15">
@@ -15761,8 +15972,8 @@
       <c r="D802" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E802" s="7" t="s">
-        <v>375</v>
+      <c r="E802" s="12" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="803" spans="1:5" ht="15">
@@ -17038,6 +17249,3100 @@
       </c>
       <c r="E877" s="2" t="s">
         <v>368</v>
+      </c>
+    </row>
+    <row r="878" spans="1:5" ht="15">
+      <c r="A878" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="B878" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C878" t="s">
+        <v>2</v>
+      </c>
+      <c r="D878" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E878" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="879" spans="1:5" ht="15">
+      <c r="A879" s="11" t="s">
+        <v>442</v>
+      </c>
+      <c r="B879" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C879" t="s">
+        <v>2</v>
+      </c>
+      <c r="D879" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E879" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="880" spans="1:5" ht="15">
+      <c r="A880" s="11" t="s">
+        <v>443</v>
+      </c>
+      <c r="B880" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C880" t="s">
+        <v>2</v>
+      </c>
+      <c r="D880" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E880" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="881" spans="1:5" ht="15">
+      <c r="A881" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="B881" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C881" t="s">
+        <v>2</v>
+      </c>
+      <c r="D881" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E881" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="882" spans="1:5" ht="15">
+      <c r="A882" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="B882" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C882" t="s">
+        <v>2</v>
+      </c>
+      <c r="D882" t="s">
+        <v>3</v>
+      </c>
+      <c r="E882" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="883" spans="1:5" ht="15">
+      <c r="A883" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B883" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C883" t="s">
+        <v>2</v>
+      </c>
+      <c r="D883" t="s">
+        <v>6</v>
+      </c>
+      <c r="E883" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="884" spans="1:5" ht="15">
+      <c r="A884" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B884" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C884" t="s">
+        <v>2</v>
+      </c>
+      <c r="D884" t="s">
+        <v>3</v>
+      </c>
+      <c r="E884" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="885" spans="1:5" ht="15">
+      <c r="A885" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B885" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C885" t="s">
+        <v>2</v>
+      </c>
+      <c r="D885" t="s">
+        <v>6</v>
+      </c>
+      <c r="E885" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="886" spans="1:5" ht="15">
+      <c r="A886" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B886" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C886" t="s">
+        <v>2</v>
+      </c>
+      <c r="D886" t="s">
+        <v>3</v>
+      </c>
+      <c r="E886" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="887" spans="1:5" ht="15">
+      <c r="A887" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="B887" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C887" t="s">
+        <v>2</v>
+      </c>
+      <c r="D887" t="s">
+        <v>3</v>
+      </c>
+      <c r="E887" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="888" spans="1:5" ht="15">
+      <c r="A888" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="B888" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C888" t="s">
+        <v>2</v>
+      </c>
+      <c r="D888" t="s">
+        <v>6</v>
+      </c>
+      <c r="E888" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="889" spans="1:5" ht="15">
+      <c r="A889" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="B889" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C889" t="s">
+        <v>2</v>
+      </c>
+      <c r="D889" t="s">
+        <v>3</v>
+      </c>
+      <c r="E889" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="890" spans="1:5" ht="77">
+      <c r="A890" s="13" t="s">
+        <v>531</v>
+      </c>
+      <c r="B890" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C890" t="s">
+        <v>2</v>
+      </c>
+      <c r="D890" t="s">
+        <v>6</v>
+      </c>
+      <c r="E890" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="891" spans="1:5" ht="77">
+      <c r="A891" s="13" t="s">
+        <v>532</v>
+      </c>
+      <c r="B891" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C891" t="s">
+        <v>2</v>
+      </c>
+      <c r="D891" t="s">
+        <v>6</v>
+      </c>
+      <c r="E891" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="892" spans="1:5" ht="15">
+      <c r="A892" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="B892" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C892" t="s">
+        <v>2</v>
+      </c>
+      <c r="D892" t="s">
+        <v>6</v>
+      </c>
+      <c r="E892" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="893" spans="1:5" ht="15">
+      <c r="A893" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="B893" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C893" t="s">
+        <v>2</v>
+      </c>
+      <c r="D893" t="s">
+        <v>3</v>
+      </c>
+      <c r="E893" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="894" spans="1:5" ht="15">
+      <c r="A894" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="B894" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C894" t="s">
+        <v>2</v>
+      </c>
+      <c r="D894" t="s">
+        <v>6</v>
+      </c>
+      <c r="E894" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="895" spans="1:5" ht="15">
+      <c r="A895" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="B895" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C895" t="s">
+        <v>2</v>
+      </c>
+      <c r="D895" t="s">
+        <v>6</v>
+      </c>
+      <c r="E895" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="896" spans="1:5" ht="77">
+      <c r="A896" s="13" t="s">
+        <v>537</v>
+      </c>
+      <c r="B896" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C896" t="s">
+        <v>2</v>
+      </c>
+      <c r="D896" t="s">
+        <v>6</v>
+      </c>
+      <c r="E896" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="897" spans="1:5" ht="77">
+      <c r="A897" s="13" t="s">
+        <v>538</v>
+      </c>
+      <c r="B897" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C897" t="s">
+        <v>2</v>
+      </c>
+      <c r="D897" t="s">
+        <v>6</v>
+      </c>
+      <c r="E897" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="898" spans="1:5" ht="15">
+      <c r="A898" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="B898" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C898" t="s">
+        <v>2</v>
+      </c>
+      <c r="D898" t="s">
+        <v>6</v>
+      </c>
+      <c r="E898" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="899" spans="1:5" ht="15">
+      <c r="A899" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="B899" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C899" t="s">
+        <v>2</v>
+      </c>
+      <c r="D899" t="s">
+        <v>42</v>
+      </c>
+      <c r="E899" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="900" spans="1:5" ht="15">
+      <c r="A900" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B900" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C900" t="s">
+        <v>2</v>
+      </c>
+      <c r="D900" t="s">
+        <v>31</v>
+      </c>
+      <c r="E900" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="901" spans="1:5" ht="15">
+      <c r="A901" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B901" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C901" t="s">
+        <v>29</v>
+      </c>
+      <c r="D901" t="s">
+        <v>192</v>
+      </c>
+      <c r="E901" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="902" spans="1:5" ht="15">
+      <c r="A902" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B902" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C902" t="s">
+        <v>29</v>
+      </c>
+      <c r="D902" t="s">
+        <v>6</v>
+      </c>
+      <c r="E902" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="903" spans="1:5" ht="15">
+      <c r="A903" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B903" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C903" t="s">
+        <v>29</v>
+      </c>
+      <c r="D903" t="s">
+        <v>3</v>
+      </c>
+      <c r="E903" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="904" spans="1:5" ht="15">
+      <c r="A904" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B904" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C904" t="s">
+        <v>29</v>
+      </c>
+      <c r="D904" t="s">
+        <v>3</v>
+      </c>
+      <c r="E904" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="905" spans="1:5" ht="15">
+      <c r="A905" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B905" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C905" t="s">
+        <v>29</v>
+      </c>
+      <c r="D905" t="s">
+        <v>3</v>
+      </c>
+      <c r="E905" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="906" spans="1:5" ht="15">
+      <c r="A906" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="B906" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C906" t="s">
+        <v>29</v>
+      </c>
+      <c r="D906" t="s">
+        <v>3</v>
+      </c>
+      <c r="E906" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="907" spans="1:5">
+      <c r="A907" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B907" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C907" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D907" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E907" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="908" spans="1:5">
+      <c r="A908" s="14" t="s">
+        <v>543</v>
+      </c>
+      <c r="B908" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C908" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D908" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E908" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="909" spans="1:5">
+      <c r="A909" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B909" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C909" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D909" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E909" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="910" spans="1:5">
+      <c r="A910" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B910" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C910" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D910" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E910" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="911" spans="1:5">
+      <c r="A911" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B911" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C911" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D911" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E911" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="912" spans="1:5">
+      <c r="A912" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B912" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C912" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D912" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E912" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="913" spans="1:5">
+      <c r="A913" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B913" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C913" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D913" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E913" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="914" spans="1:5">
+      <c r="A914" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B914" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C914" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D914" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E914" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="915" spans="1:5">
+      <c r="A915" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B915" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C915" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D915" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E915" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="916" spans="1:5">
+      <c r="A916" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B916" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C916" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D916" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E916" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="917" spans="1:5">
+      <c r="A917" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B917" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C917" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D917" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E917" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="918" spans="1:5">
+      <c r="A918" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B918" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C918" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D918" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E918" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="919" spans="1:5">
+      <c r="A919" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B919" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C919" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D919" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E919" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="920" spans="1:5">
+      <c r="A920" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B920" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C920" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D920" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E920" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="921" spans="1:5">
+      <c r="A921" s="14" t="s">
+        <v>543</v>
+      </c>
+      <c r="B921" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C921" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D921" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E921" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="922" spans="1:5">
+      <c r="A922" s="14" t="s">
+        <v>543</v>
+      </c>
+      <c r="B922" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C922" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D922" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E922" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="923" spans="1:5">
+      <c r="A923" s="14" t="s">
+        <v>543</v>
+      </c>
+      <c r="B923" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C923" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D923" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E923" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="924" spans="1:5">
+      <c r="A924" s="14" t="s">
+        <v>543</v>
+      </c>
+      <c r="B924" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C924" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D924" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E924" s="18" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="925" spans="1:5">
+      <c r="A925" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B925" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C925" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D925" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E925" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="926" spans="1:5">
+      <c r="A926" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B926" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C926" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D926" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E926" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="927" spans="1:5">
+      <c r="A927" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B927" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C927" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D927" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E927" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="928" spans="1:5">
+      <c r="A928" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B928" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C928" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D928" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E928" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="929" spans="1:5">
+      <c r="A929" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B929" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C929" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D929" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E929" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="930" spans="1:5">
+      <c r="A930" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B930" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C930" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D930" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E930" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="931" spans="1:5">
+      <c r="A931" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B931" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C931" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D931" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E931" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="932" spans="1:5">
+      <c r="A932" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B932" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C932" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D932" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E932" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="933" spans="1:5">
+      <c r="A933" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B933" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C933" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D933" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E933" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="934" spans="1:5">
+      <c r="A934" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B934" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C934" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D934" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E934" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="935" spans="1:5">
+      <c r="A935" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B935" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C935" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D935" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E935" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="936" spans="1:5">
+      <c r="A936" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B936" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C936" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D936" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E936" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="937" spans="1:5">
+      <c r="A937" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B937" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C937" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D937" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E937" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="938" spans="1:5">
+      <c r="A938" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B938" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C938" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D938" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E938" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="939" spans="1:5">
+      <c r="A939" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B939" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C939" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D939" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E939" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="940" spans="1:5">
+      <c r="A940" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B940" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C940" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D940" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E940" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="941" spans="1:5">
+      <c r="A941" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B941" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C941" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D941" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E941" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="942" spans="1:5">
+      <c r="A942" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B942" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C942" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D942" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E942" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="943" spans="1:5">
+      <c r="A943" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B943" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C943" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D943" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E943" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="944" spans="1:5">
+      <c r="A944" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B944" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C944" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D944" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E944" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="945" spans="1:5">
+      <c r="A945" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B945" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C945" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D945" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E945" s="16" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="946" spans="1:5">
+      <c r="A946" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="B946" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C946" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D946" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E946" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="947" spans="1:5">
+      <c r="A947" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B947" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C947" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D947" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E947" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="948" spans="1:5">
+      <c r="A948" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B948" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C948" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D948" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E948" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="949" spans="1:5">
+      <c r="A949" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="B949" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C949" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D949" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E949" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="950" spans="1:5">
+      <c r="A950" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="B950" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C950" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D950" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E950" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="951" spans="1:5">
+      <c r="A951" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="B951" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C951" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D951" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E951" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="952" spans="1:5">
+      <c r="A952" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B952" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C952" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D952" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E952" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="953" spans="1:5">
+      <c r="A953" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B953" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C953" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D953" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E953" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="954" spans="1:5">
+      <c r="A954" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B954" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C954" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D954" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E954" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="955" spans="1:5">
+      <c r="A955" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B955" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C955" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D955" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E955" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="956" spans="1:5">
+      <c r="A956" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B956" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C956" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D956" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E956" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="957" spans="1:5">
+      <c r="A957" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="B957" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C957" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D957" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E957" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="958" spans="1:5">
+      <c r="A958" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B958" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C958" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D958" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E958" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="959" spans="1:5">
+      <c r="A959" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B959" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C959" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D959" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E959" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="960" spans="1:5">
+      <c r="A960" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B960" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C960" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D960" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E960" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="961" spans="1:5">
+      <c r="A961" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B961" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C961" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D961" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E961" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="962" spans="1:5">
+      <c r="A962" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B962" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C962" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D962" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E962" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="963" spans="1:5">
+      <c r="A963" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B963" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C963" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D963" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E963" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="964" spans="1:5">
+      <c r="A964" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B964" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C964" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D964" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E964" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="965" spans="1:5">
+      <c r="A965" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B965" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C965" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D965" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E965" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="966" spans="1:5">
+      <c r="A966" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B966" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C966" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D966" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E966" s="16" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="967" spans="1:5">
+      <c r="A967" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B967" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C967" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D967" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E967" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="968" spans="1:5">
+      <c r="A968" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B968" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C968" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D968" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E968" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="969" spans="1:5">
+      <c r="A969" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B969" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C969" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D969" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E969" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="970" spans="1:5">
+      <c r="A970" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B970" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C970" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D970" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E970" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="971" spans="1:5">
+      <c r="A971" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B971" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C971" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D971" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E971" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="972" spans="1:5">
+      <c r="A972" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B972" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C972" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D972" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E972" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="973" spans="1:5">
+      <c r="A973" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B973" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C973" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D973" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E973" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="974" spans="1:5">
+      <c r="A974" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B974" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C974" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D974" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E974" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="975" spans="1:5">
+      <c r="A975" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B975" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C975" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D975" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E975" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="976" spans="1:5">
+      <c r="A976" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B976" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C976" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D976" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E976" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="977" spans="1:5">
+      <c r="A977" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B977" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C977" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D977" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E977" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="978" spans="1:5">
+      <c r="A978" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B978" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C978" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D978" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E978" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="979" spans="1:5">
+      <c r="A979" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B979" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C979" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D979" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E979" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="980" spans="1:5">
+      <c r="A980" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B980" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C980" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D980" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E980" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="981" spans="1:5">
+      <c r="A981" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B981" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C981" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D981" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E981" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="982" spans="1:5">
+      <c r="A982" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B982" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C982" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D982" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E982" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="983" spans="1:5">
+      <c r="A983" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B983" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C983" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D983" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E983" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="984" spans="1:5">
+      <c r="A984" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B984" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C984" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D984" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E984" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="985" spans="1:5">
+      <c r="A985" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B985" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C985" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D985" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E985" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="986" spans="1:5">
+      <c r="A986" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B986" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C986" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D986" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E986" s="16" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="987" spans="1:5">
+      <c r="A987" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B987" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C987" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D987" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E987" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="988" spans="1:5">
+      <c r="A988" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B988" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C988" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D988" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E988" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="989" spans="1:5">
+      <c r="A989" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B989" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C989" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D989" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E989" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="990" spans="1:5">
+      <c r="A990" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B990" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C990" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D990" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E990" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="991" spans="1:5">
+      <c r="A991" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B991" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C991" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D991" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E991" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="992" spans="1:5">
+      <c r="A992" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B992" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C992" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D992" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E992" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="993" spans="1:5">
+      <c r="A993" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B993" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C993" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D993" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E993" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="994" spans="1:5">
+      <c r="A994" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B994" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C994" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D994" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E994" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="995" spans="1:5">
+      <c r="A995" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B995" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C995" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D995" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E995" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="996" spans="1:5">
+      <c r="A996" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B996" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C996" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D996" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E996" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="997" spans="1:5">
+      <c r="A997" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B997" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C997" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D997" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E997" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="998" spans="1:5">
+      <c r="A998" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B998" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C998" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D998" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E998" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="999" spans="1:5">
+      <c r="A999" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B999" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C999" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D999" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E999" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:5">
+      <c r="A1000" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B1000" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1000" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1000" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1000" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:5">
+      <c r="A1001" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="B1001" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1001" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1001" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1001" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:5">
+      <c r="A1002" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1002" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1002" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1002" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1002" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:5">
+      <c r="A1003" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1003" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1003" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1003" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1003" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:5">
+      <c r="A1004" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1004" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1004" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1004" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1004" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:5">
+      <c r="A1005" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1005" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1005" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1005" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1005" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:5">
+      <c r="A1006" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1006" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1006" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1006" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1006" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:5">
+      <c r="A1007" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1007" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1007" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1007" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1007" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:5">
+      <c r="A1008" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="B1008" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1008" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1008" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1008" s="16" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:5">
+      <c r="A1009" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B1009" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1009" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1009" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1009" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:5">
+      <c r="A1010" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1010" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1010" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1010" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1010" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:5">
+      <c r="A1011" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B1011" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1011" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1011" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1011" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:5">
+      <c r="A1012" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1012" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1012" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1012" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1012" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:5">
+      <c r="A1013" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1013" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1013" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1013" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1013" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:5">
+      <c r="A1014" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1014" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1014" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1014" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1014" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:5">
+      <c r="A1015" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1015" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1015" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1015" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1015" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:5">
+      <c r="A1016" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1016" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1016" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1016" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1016" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:5">
+      <c r="A1017" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B1017" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1017" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1017" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1017" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:5">
+      <c r="A1018" s="14" t="s">
+        <v>544</v>
+      </c>
+      <c r="B1018" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1018" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1018" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1018" s="16" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:5" ht="15">
+      <c r="A1019" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B1019" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1019" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1019" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1019" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:5" ht="15">
+      <c r="A1020" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B1020" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1020" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1020" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1020" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:5" ht="15">
+      <c r="A1021" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="B1021" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1021" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1021" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1021" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:5" ht="15">
+      <c r="A1022" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="B1022" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1022" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1022" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="E1022" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:5" ht="15">
+      <c r="A1023" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1023" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1023" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1023" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1023" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:5" ht="15">
+      <c r="A1024" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="B1024" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1024" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1024" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1024" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:5" ht="15">
+      <c r="A1025" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="B1025" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1025" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1025" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1025" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:5" ht="15">
+      <c r="A1026" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="B1026" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1026" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1026" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1026" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:5" ht="15">
+      <c r="A1027" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="B1027" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1027" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1027" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1027" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:5" ht="15">
+      <c r="A1028" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="B1028" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1028" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1028" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1028" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:5" ht="15">
+      <c r="A1029" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="B1029" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1029" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1029" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1029" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:5" ht="15">
+      <c r="A1030" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="B1030" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1030" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1030" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1030" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:5" ht="15">
+      <c r="A1031" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="B1031" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1031" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1031" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1031" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:5" ht="15">
+      <c r="A1032" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="B1032" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1032" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1032" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1032" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:5" ht="15">
+      <c r="A1033" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="B1033" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1033" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1033" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1033" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:5" ht="15">
+      <c r="A1034" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="B1034" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1034" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1034" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1034" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:5" ht="15">
+      <c r="A1035" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="B1035" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1035" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1035" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1035" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:5" ht="15">
+      <c r="A1036" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="B1036" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1036" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1036" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1036" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:5" ht="15">
+      <c r="A1037" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="B1037" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1037" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1037" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1037" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:5" ht="15">
+      <c r="A1038" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="B1038" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1038" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1038" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1038" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:5" ht="15">
+      <c r="A1039" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="B1039" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1039" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1039" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1039" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:5" ht="15">
+      <c r="A1040" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="B1040" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1040" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1040" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1040" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:5" ht="15">
+      <c r="A1041" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="B1041" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1041" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1041" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1041" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:5" ht="15">
+      <c r="A1042" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1042" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1042" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1042" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1042" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:5" ht="15">
+      <c r="A1043" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="B1043" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C1043" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1043" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1043" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:5" ht="15">
+      <c r="A1044" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="B1044" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1044" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1044" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1044" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:5" ht="15">
+      <c r="A1045" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="B1045" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1045" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1045" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1045" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:5" ht="15">
+      <c r="A1046" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="B1046" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1046" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1046" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1046" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:5" ht="15">
+      <c r="A1047" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="B1047" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1047" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1047" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1047" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:5" ht="15">
+      <c r="A1048" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="B1048" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1048" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1048" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1048" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:5" ht="15">
+      <c r="A1049" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="B1049" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1049" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1049" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1049" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1050" spans="1:5" ht="15">
+      <c r="A1050" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="B1050" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1050" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1050" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1050" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1051" spans="1:5" ht="15">
+      <c r="A1051" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="B1051" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1051" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1051" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1051" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1052" spans="1:5" ht="15">
+      <c r="A1052" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="B1052" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1052" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1052" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1052" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1053" spans="1:5" ht="15">
+      <c r="A1053" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="B1053" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1053" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1053" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1053" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1054" spans="1:5" ht="15">
+      <c r="A1054" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="B1054" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1054" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1054" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1054" s="16" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1055" spans="1:5" ht="15">
+      <c r="A1055" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="B1055" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1055" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1055" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1055" s="20" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1056" spans="1:5" ht="15">
+      <c r="A1056" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1056" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1056" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1056" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1056" s="20" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:5" ht="15">
+      <c r="A1057" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1057" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1057" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1057" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1057" s="20" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:5" ht="15">
+      <c r="A1058" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1058" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1058" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1058" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1058" s="20" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:5" ht="15">
+      <c r="A1059" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="B1059" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1059" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1059" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1059" s="2" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FBB basic land pricing references
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B261438-5604-44A6-84E2-9DF90693E1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B05A57-1855-4644-AF4F-2FBA94DB0B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5295" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5300" uniqueCount="584">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -1925,7 +1925,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1962,28 +1962,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2333,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E1059"/>
+  <dimension ref="A1:E1060"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -17745,1906 +17733,1906 @@
       </c>
     </row>
     <row r="907" spans="1:5">
-      <c r="A907" s="14" t="s">
+      <c r="A907" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B907" s="15" t="s">
+      <c r="B907" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C907" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D907" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E907" s="16" t="s">
+      <c r="C907" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D907" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E907" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="908" spans="1:5">
-      <c r="A908" s="14" t="s">
+      <c r="A908" s="9" t="s">
         <v>543</v>
       </c>
-      <c r="B908" s="15" t="s">
+      <c r="B908" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C908" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D908" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E908" s="16" t="s">
+      <c r="C908" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D908" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E908" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="909" spans="1:5">
-      <c r="A909" s="14" t="s">
+      <c r="A909" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B909" s="15" t="s">
+      <c r="B909" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C909" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D909" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E909" s="18" t="s">
+      <c r="C909" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D909" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E909" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="910" spans="1:5">
-      <c r="A910" s="14" t="s">
+      <c r="A910" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B910" s="15" t="s">
+      <c r="B910" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C910" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D910" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E910" s="18" t="s">
+      <c r="C910" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D910" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E910" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="911" spans="1:5">
-      <c r="A911" s="14" t="s">
+      <c r="A911" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B911" s="15" t="s">
+      <c r="B911" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C911" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D911" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E911" s="18" t="s">
+      <c r="C911" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D911" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E911" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="912" spans="1:5">
-      <c r="A912" s="14" t="s">
+      <c r="A912" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B912" s="15" t="s">
+      <c r="B912" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C912" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D912" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E912" s="18" t="s">
+      <c r="C912" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D912" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E912" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="913" spans="1:5">
-      <c r="A913" s="14" t="s">
+      <c r="A913" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B913" s="15" t="s">
+      <c r="B913" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C913" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D913" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E913" s="18" t="s">
+      <c r="C913" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D913" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E913" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="914" spans="1:5">
-      <c r="A914" s="14" t="s">
+      <c r="A914" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B914" s="15" t="s">
+      <c r="B914" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C914" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D914" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E914" s="18" t="s">
+      <c r="C914" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D914" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E914" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="915" spans="1:5">
-      <c r="A915" s="14" t="s">
+      <c r="A915" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B915" s="15" t="s">
+      <c r="B915" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C915" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D915" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E915" s="18" t="s">
+      <c r="C915" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D915" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E915" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="916" spans="1:5">
-      <c r="A916" s="14" t="s">
+      <c r="A916" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B916" s="15" t="s">
+      <c r="B916" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C916" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D916" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E916" s="18" t="s">
+      <c r="C916" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D916" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E916" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="917" spans="1:5">
-      <c r="A917" s="14" t="s">
+      <c r="A917" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B917" s="15" t="s">
+      <c r="B917" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C917" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D917" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E917" s="18" t="s">
+      <c r="C917" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D917" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E917" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="918" spans="1:5">
-      <c r="A918" s="14" t="s">
+      <c r="A918" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B918" s="15" t="s">
+      <c r="B918" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C918" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D918" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E918" s="18" t="s">
+      <c r="C918" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D918" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E918" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="919" spans="1:5">
-      <c r="A919" s="14" t="s">
+      <c r="A919" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B919" s="15" t="s">
+      <c r="B919" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C919" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D919" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E919" s="18" t="s">
+      <c r="C919" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D919" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E919" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="920" spans="1:5">
-      <c r="A920" s="14" t="s">
+      <c r="A920" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B920" s="15" t="s">
+      <c r="B920" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C920" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D920" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E920" s="18" t="s">
+      <c r="C920" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D920" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E920" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="921" spans="1:5">
-      <c r="A921" s="14" t="s">
+      <c r="A921" s="9" t="s">
         <v>543</v>
       </c>
-      <c r="B921" s="15" t="s">
+      <c r="B921" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C921" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D921" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E921" s="18" t="s">
+      <c r="C921" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D921" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E921" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="922" spans="1:5">
-      <c r="A922" s="14" t="s">
+      <c r="A922" s="9" t="s">
         <v>543</v>
       </c>
-      <c r="B922" s="15" t="s">
+      <c r="B922" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C922" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D922" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E922" s="18" t="s">
+      <c r="C922" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D922" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E922" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="923" spans="1:5">
-      <c r="A923" s="14" t="s">
+      <c r="A923" s="9" t="s">
         <v>543</v>
       </c>
-      <c r="B923" s="15" t="s">
+      <c r="B923" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C923" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D923" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E923" s="18" t="s">
+      <c r="C923" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D923" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E923" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="924" spans="1:5">
-      <c r="A924" s="14" t="s">
+      <c r="A924" s="9" t="s">
         <v>543</v>
       </c>
-      <c r="B924" s="15" t="s">
+      <c r="B924" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C924" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D924" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E924" s="18" t="s">
+      <c r="C924" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D924" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E924" s="2" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="925" spans="1:5">
-      <c r="A925" s="14" t="s">
+      <c r="A925" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B925" s="15" t="s">
+      <c r="B925" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C925" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D925" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E925" s="16" t="s">
+      <c r="C925" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D925" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E925" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="926" spans="1:5">
-      <c r="A926" s="14" t="s">
+      <c r="A926" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B926" s="15" t="s">
+      <c r="B926" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C926" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D926" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E926" s="16" t="s">
+      <c r="C926" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D926" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E926" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="927" spans="1:5">
-      <c r="A927" s="14" t="s">
+      <c r="A927" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B927" s="15" t="s">
+      <c r="B927" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C927" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D927" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E927" s="16" t="s">
+      <c r="C927" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D927" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E927" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="928" spans="1:5">
-      <c r="A928" s="14" t="s">
+      <c r="A928" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B928" s="15" t="s">
+      <c r="B928" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C928" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D928" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E928" s="16" t="s">
+      <c r="C928" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D928" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E928" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="929" spans="1:5">
-      <c r="A929" s="14" t="s">
+      <c r="A929" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B929" s="15" t="s">
+      <c r="B929" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C929" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D929" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E929" s="16" t="s">
+      <c r="C929" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D929" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E929" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="930" spans="1:5">
-      <c r="A930" s="14" t="s">
+      <c r="A930" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B930" s="15" t="s">
+      <c r="B930" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C930" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D930" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E930" s="16" t="s">
+      <c r="C930" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D930" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E930" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="931" spans="1:5">
-      <c r="A931" s="14" t="s">
+      <c r="A931" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B931" s="15" t="s">
+      <c r="B931" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C931" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D931" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E931" s="16" t="s">
+      <c r="C931" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D931" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E931" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="932" spans="1:5">
-      <c r="A932" s="14" t="s">
+      <c r="A932" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B932" s="15" t="s">
+      <c r="B932" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C932" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D932" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E932" s="16" t="s">
+      <c r="C932" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D932" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E932" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="933" spans="1:5">
-      <c r="A933" s="14" t="s">
+      <c r="A933" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B933" s="15" t="s">
+      <c r="B933" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C933" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D933" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E933" s="16" t="s">
+      <c r="C933" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D933" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E933" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="934" spans="1:5">
-      <c r="A934" s="14" t="s">
+      <c r="A934" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B934" s="15" t="s">
+      <c r="B934" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C934" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D934" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E934" s="16" t="s">
+      <c r="C934" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D934" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E934" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="935" spans="1:5">
-      <c r="A935" s="14" t="s">
+      <c r="A935" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B935" s="15" t="s">
+      <c r="B935" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C935" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D935" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E935" s="16" t="s">
+      <c r="C935" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D935" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E935" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="936" spans="1:5">
-      <c r="A936" s="14" t="s">
+      <c r="A936" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B936" s="15" t="s">
+      <c r="B936" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C936" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D936" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E936" s="16" t="s">
+      <c r="C936" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D936" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E936" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="937" spans="1:5">
-      <c r="A937" s="14" t="s">
+      <c r="A937" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B937" s="15" t="s">
+      <c r="B937" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C937" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D937" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E937" s="16" t="s">
+      <c r="C937" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D937" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E937" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="938" spans="1:5">
-      <c r="A938" s="14" t="s">
+      <c r="A938" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B938" s="15" t="s">
+      <c r="B938" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C938" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D938" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E938" s="16" t="s">
+      <c r="C938" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D938" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E938" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="939" spans="1:5">
-      <c r="A939" s="14" t="s">
+      <c r="A939" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B939" s="15" t="s">
+      <c r="B939" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C939" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D939" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E939" s="16" t="s">
+      <c r="C939" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D939" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E939" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="940" spans="1:5">
-      <c r="A940" s="14" t="s">
+      <c r="A940" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B940" s="15" t="s">
+      <c r="B940" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C940" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D940" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E940" s="16" t="s">
+      <c r="C940" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D940" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E940" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="941" spans="1:5">
-      <c r="A941" s="14" t="s">
+      <c r="A941" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B941" s="15" t="s">
+      <c r="B941" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C941" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D941" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E941" s="16" t="s">
+      <c r="C941" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D941" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E941" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="942" spans="1:5">
-      <c r="A942" s="14" t="s">
+      <c r="A942" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B942" s="15" t="s">
+      <c r="B942" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C942" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D942" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E942" s="16" t="s">
+      <c r="C942" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D942" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E942" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="943" spans="1:5">
-      <c r="A943" s="14" t="s">
+      <c r="A943" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B943" s="15" t="s">
+      <c r="B943" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C943" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D943" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E943" s="16" t="s">
+      <c r="C943" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D943" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E943" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="944" spans="1:5">
-      <c r="A944" s="14" t="s">
+      <c r="A944" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B944" s="15" t="s">
+      <c r="B944" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C944" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D944" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E944" s="16" t="s">
+      <c r="C944" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D944" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E944" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="945" spans="1:5">
-      <c r="A945" s="14" t="s">
+      <c r="A945" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B945" s="15" t="s">
+      <c r="B945" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C945" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D945" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E945" s="16" t="s">
+      <c r="C945" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D945" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E945" s="10" t="s">
         <v>374</v>
       </c>
     </row>
     <row r="946" spans="1:5">
-      <c r="A946" s="19" t="s">
+      <c r="A946" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="B946" s="15" t="s">
+      <c r="B946" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C946" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D946" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E946" s="16" t="s">
+      <c r="C946" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D946" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E946" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="947" spans="1:5">
-      <c r="A947" s="19" t="s">
+      <c r="A947" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B947" s="15" t="s">
+      <c r="B947" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C947" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D947" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E947" s="16" t="s">
+      <c r="C947" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D947" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E947" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="948" spans="1:5">
-      <c r="A948" s="19" t="s">
+      <c r="A948" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B948" s="15" t="s">
+      <c r="B948" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C948" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D948" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E948" s="16" t="s">
+      <c r="C948" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D948" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E948" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="949" spans="1:5">
-      <c r="A949" s="19" t="s">
+      <c r="A949" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="B949" s="15" t="s">
+      <c r="B949" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C949" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D949" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E949" s="16" t="s">
+      <c r="C949" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D949" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E949" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="950" spans="1:5">
-      <c r="A950" s="19" t="s">
+      <c r="A950" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="B950" s="15" t="s">
+      <c r="B950" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C950" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D950" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E950" s="16" t="s">
+      <c r="C950" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D950" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E950" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="951" spans="1:5">
-      <c r="A951" s="19" t="s">
+      <c r="A951" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="B951" s="15" t="s">
+      <c r="B951" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C951" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D951" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E951" s="16" t="s">
+      <c r="C951" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D951" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E951" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="952" spans="1:5">
-      <c r="A952" s="19" t="s">
+      <c r="A952" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B952" s="15" t="s">
+      <c r="B952" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C952" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D952" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E952" s="16" t="s">
+      <c r="C952" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D952" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E952" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="953" spans="1:5">
-      <c r="A953" s="19" t="s">
+      <c r="A953" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B953" s="15" t="s">
+      <c r="B953" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C953" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D953" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E953" s="16" t="s">
+      <c r="C953" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D953" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E953" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="954" spans="1:5">
-      <c r="A954" s="19" t="s">
+      <c r="A954" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B954" s="15" t="s">
+      <c r="B954" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C954" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D954" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E954" s="16" t="s">
+      <c r="C954" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D954" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E954" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="955" spans="1:5">
-      <c r="A955" s="19" t="s">
+      <c r="A955" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B955" s="15" t="s">
+      <c r="B955" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C955" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D955" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E955" s="16" t="s">
+      <c r="C955" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D955" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E955" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="956" spans="1:5">
-      <c r="A956" s="19" t="s">
+      <c r="A956" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B956" s="15" t="s">
+      <c r="B956" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C956" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D956" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E956" s="16" t="s">
+      <c r="C956" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D956" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E956" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="957" spans="1:5">
-      <c r="A957" s="19" t="s">
+      <c r="A957" s="14" t="s">
         <v>545</v>
       </c>
-      <c r="B957" s="15" t="s">
+      <c r="B957" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C957" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D957" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E957" s="16" t="s">
+      <c r="C957" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D957" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E957" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="958" spans="1:5">
-      <c r="A958" s="19" t="s">
+      <c r="A958" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B958" s="15" t="s">
+      <c r="B958" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C958" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D958" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E958" s="16" t="s">
+      <c r="C958" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D958" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E958" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="959" spans="1:5">
-      <c r="A959" s="19" t="s">
+      <c r="A959" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B959" s="15" t="s">
+      <c r="B959" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C959" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D959" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E959" s="16" t="s">
+      <c r="C959" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D959" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E959" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="960" spans="1:5">
-      <c r="A960" s="19" t="s">
+      <c r="A960" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B960" s="15" t="s">
+      <c r="B960" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C960" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D960" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E960" s="16" t="s">
+      <c r="C960" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D960" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E960" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="961" spans="1:5">
-      <c r="A961" s="19" t="s">
+      <c r="A961" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B961" s="15" t="s">
+      <c r="B961" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C961" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D961" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E961" s="16" t="s">
+      <c r="C961" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D961" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E961" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="962" spans="1:5">
-      <c r="A962" s="19" t="s">
+      <c r="A962" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B962" s="15" t="s">
+      <c r="B962" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C962" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D962" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E962" s="16" t="s">
+      <c r="C962" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D962" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E962" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="963" spans="1:5">
-      <c r="A963" s="19" t="s">
+      <c r="A963" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B963" s="15" t="s">
+      <c r="B963" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C963" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D963" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E963" s="16" t="s">
+      <c r="C963" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D963" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E963" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="964" spans="1:5">
-      <c r="A964" s="19" t="s">
+      <c r="A964" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B964" s="15" t="s">
+      <c r="B964" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C964" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D964" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E964" s="16" t="s">
+      <c r="C964" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D964" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E964" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="965" spans="1:5">
-      <c r="A965" s="19" t="s">
+      <c r="A965" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B965" s="15" t="s">
+      <c r="B965" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C965" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D965" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E965" s="16" t="s">
+      <c r="C965" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D965" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E965" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="966" spans="1:5">
-      <c r="A966" s="19" t="s">
+      <c r="A966" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B966" s="15" t="s">
+      <c r="B966" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C966" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D966" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E966" s="16" t="s">
+      <c r="C966" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D966" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E966" s="10" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="967" spans="1:5">
-      <c r="A967" s="19" t="s">
+      <c r="A967" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B967" s="15" t="s">
+      <c r="B967" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C967" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D967" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E967" s="16" t="s">
+      <c r="C967" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D967" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E967" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="968" spans="1:5">
-      <c r="A968" s="19" t="s">
+      <c r="A968" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B968" s="15" t="s">
+      <c r="B968" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C968" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D968" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E968" s="16" t="s">
+      <c r="C968" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D968" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E968" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="969" spans="1:5">
-      <c r="A969" s="19" t="s">
+      <c r="A969" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B969" s="15" t="s">
+      <c r="B969" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C969" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D969" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E969" s="16" t="s">
+      <c r="C969" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D969" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E969" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="970" spans="1:5">
-      <c r="A970" s="19" t="s">
+      <c r="A970" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B970" s="15" t="s">
+      <c r="B970" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C970" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D970" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E970" s="16" t="s">
+      <c r="C970" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D970" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E970" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="971" spans="1:5">
-      <c r="A971" s="19" t="s">
+      <c r="A971" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B971" s="15" t="s">
+      <c r="B971" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C971" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D971" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E971" s="16" t="s">
+      <c r="C971" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D971" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E971" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="972" spans="1:5">
-      <c r="A972" s="19" t="s">
+      <c r="A972" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B972" s="15" t="s">
+      <c r="B972" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C972" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D972" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E972" s="16" t="s">
+      <c r="C972" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D972" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E972" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="973" spans="1:5">
-      <c r="A973" s="19" t="s">
+      <c r="A973" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B973" s="15" t="s">
+      <c r="B973" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C973" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D973" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E973" s="16" t="s">
+      <c r="C973" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D973" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E973" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="974" spans="1:5">
-      <c r="A974" s="19" t="s">
+      <c r="A974" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B974" s="15" t="s">
+      <c r="B974" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C974" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D974" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E974" s="16" t="s">
+      <c r="C974" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D974" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E974" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="975" spans="1:5">
-      <c r="A975" s="19" t="s">
+      <c r="A975" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B975" s="15" t="s">
+      <c r="B975" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C975" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D975" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E975" s="16" t="s">
+      <c r="C975" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D975" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E975" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="976" spans="1:5">
-      <c r="A976" s="19" t="s">
+      <c r="A976" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B976" s="15" t="s">
+      <c r="B976" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C976" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D976" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E976" s="16" t="s">
+      <c r="C976" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D976" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E976" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="977" spans="1:5">
-      <c r="A977" s="19" t="s">
+      <c r="A977" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B977" s="15" t="s">
+      <c r="B977" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C977" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D977" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E977" s="16" t="s">
+      <c r="C977" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D977" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E977" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="978" spans="1:5">
-      <c r="A978" s="19" t="s">
+      <c r="A978" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B978" s="15" t="s">
+      <c r="B978" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C978" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D978" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E978" s="16" t="s">
+      <c r="C978" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D978" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E978" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="979" spans="1:5">
-      <c r="A979" s="19" t="s">
+      <c r="A979" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B979" s="15" t="s">
+      <c r="B979" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C979" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D979" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E979" s="16" t="s">
+      <c r="C979" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D979" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E979" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="980" spans="1:5">
-      <c r="A980" s="19" t="s">
+      <c r="A980" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B980" s="15" t="s">
+      <c r="B980" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C980" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D980" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E980" s="16" t="s">
+      <c r="C980" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D980" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E980" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="981" spans="1:5">
-      <c r="A981" s="19" t="s">
+      <c r="A981" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B981" s="15" t="s">
+      <c r="B981" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C981" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D981" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E981" s="16" t="s">
+      <c r="C981" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D981" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E981" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="982" spans="1:5">
-      <c r="A982" s="19" t="s">
+      <c r="A982" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B982" s="15" t="s">
+      <c r="B982" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C982" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D982" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E982" s="16" t="s">
+      <c r="C982" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D982" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E982" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="983" spans="1:5">
-      <c r="A983" s="19" t="s">
+      <c r="A983" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B983" s="15" t="s">
+      <c r="B983" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C983" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D983" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E983" s="16" t="s">
+      <c r="C983" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D983" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E983" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="984" spans="1:5">
-      <c r="A984" s="19" t="s">
+      <c r="A984" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B984" s="15" t="s">
+      <c r="B984" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C984" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D984" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E984" s="16" t="s">
+      <c r="C984" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D984" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E984" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="985" spans="1:5">
-      <c r="A985" s="19" t="s">
+      <c r="A985" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B985" s="15" t="s">
+      <c r="B985" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C985" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D985" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E985" s="16" t="s">
+      <c r="C985" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D985" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E985" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="986" spans="1:5">
-      <c r="A986" s="19" t="s">
+      <c r="A986" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B986" s="15" t="s">
+      <c r="B986" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C986" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D986" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E986" s="16" t="s">
+      <c r="C986" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D986" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E986" s="10" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="987" spans="1:5">
-      <c r="A987" s="19" t="s">
+      <c r="A987" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B987" s="15" t="s">
+      <c r="B987" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C987" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D987" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E987" s="16" t="s">
+      <c r="C987" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D987" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E987" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="988" spans="1:5">
-      <c r="A988" s="19" t="s">
+      <c r="A988" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B988" s="15" t="s">
+      <c r="B988" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C988" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D988" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E988" s="16" t="s">
+      <c r="C988" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D988" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E988" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="989" spans="1:5">
-      <c r="A989" s="19" t="s">
+      <c r="A989" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B989" s="15" t="s">
+      <c r="B989" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C989" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D989" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E989" s="16" t="s">
+      <c r="C989" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D989" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E989" s="10" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="990" spans="1:5">
-      <c r="A990" s="19" t="s">
+      <c r="A990" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B990" s="15" t="s">
+      <c r="B990" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C990" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D990" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E990" s="16" t="s">
+      <c r="C990" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D990" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E990" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="991" spans="1:5">
-      <c r="A991" s="19" t="s">
+      <c r="A991" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B991" s="15" t="s">
+      <c r="B991" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C991" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D991" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E991" s="16" t="s">
+      <c r="C991" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D991" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E991" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="992" spans="1:5">
-      <c r="A992" s="19" t="s">
+      <c r="A992" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B992" s="15" t="s">
+      <c r="B992" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C992" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D992" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E992" s="16" t="s">
+      <c r="C992" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D992" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E992" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="993" spans="1:5">
-      <c r="A993" s="19" t="s">
+      <c r="A993" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B993" s="15" t="s">
+      <c r="B993" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C993" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D993" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E993" s="16" t="s">
+      <c r="C993" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D993" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E993" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="994" spans="1:5">
-      <c r="A994" s="19" t="s">
+      <c r="A994" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B994" s="15" t="s">
+      <c r="B994" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C994" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D994" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E994" s="16" t="s">
+      <c r="C994" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D994" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E994" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="995" spans="1:5">
-      <c r="A995" s="19" t="s">
+      <c r="A995" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B995" s="15" t="s">
+      <c r="B995" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C995" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D995" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E995" s="16" t="s">
+      <c r="C995" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D995" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E995" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="996" spans="1:5">
-      <c r="A996" s="19" t="s">
+      <c r="A996" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B996" s="15" t="s">
+      <c r="B996" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C996" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D996" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E996" s="16" t="s">
+      <c r="C996" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D996" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E996" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="997" spans="1:5">
-      <c r="A997" s="19" t="s">
+      <c r="A997" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B997" s="15" t="s">
+      <c r="B997" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C997" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D997" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E997" s="16" t="s">
+      <c r="C997" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D997" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E997" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="998" spans="1:5">
-      <c r="A998" s="19" t="s">
+      <c r="A998" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B998" s="15" t="s">
+      <c r="B998" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C998" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D998" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E998" s="16" t="s">
+      <c r="C998" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D998" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E998" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="999" spans="1:5">
-      <c r="A999" s="19" t="s">
+      <c r="A999" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B999" s="15" t="s">
+      <c r="B999" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C999" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D999" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E999" s="16" t="s">
+      <c r="C999" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D999" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E999" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1000" spans="1:5">
-      <c r="A1000" s="19" t="s">
+      <c r="A1000" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B1000" s="15" t="s">
+      <c r="B1000" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1000" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1000" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1000" s="16" t="s">
+      <c r="C1000" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1000" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1000" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1001" spans="1:5">
-      <c r="A1001" s="19" t="s">
+      <c r="A1001" s="14" t="s">
         <v>547</v>
       </c>
-      <c r="B1001" s="15" t="s">
+      <c r="B1001" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1001" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1001" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1001" s="16" t="s">
+      <c r="C1001" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1001" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1001" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1002" spans="1:5">
-      <c r="A1002" s="19" t="s">
+      <c r="A1002" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1002" s="15" t="s">
+      <c r="B1002" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1002" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1002" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1002" s="16" t="s">
+      <c r="C1002" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1002" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1002" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1003" spans="1:5">
-      <c r="A1003" s="19" t="s">
+      <c r="A1003" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1003" s="15" t="s">
+      <c r="B1003" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1003" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1003" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1003" s="16" t="s">
+      <c r="C1003" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1003" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1003" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1004" spans="1:5">
-      <c r="A1004" s="19" t="s">
+      <c r="A1004" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1004" s="15" t="s">
+      <c r="B1004" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1004" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1004" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1004" s="16" t="s">
+      <c r="C1004" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1004" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1004" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1005" spans="1:5">
-      <c r="A1005" s="19" t="s">
+      <c r="A1005" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1005" s="15" t="s">
+      <c r="B1005" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1005" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1005" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1005" s="16" t="s">
+      <c r="C1005" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1005" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1005" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1006" spans="1:5">
-      <c r="A1006" s="19" t="s">
+      <c r="A1006" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1006" s="15" t="s">
+      <c r="B1006" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1006" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1006" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1006" s="16" t="s">
+      <c r="C1006" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1006" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1006" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1007" spans="1:5">
-      <c r="A1007" s="19" t="s">
+      <c r="A1007" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1007" s="15" t="s">
+      <c r="B1007" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1007" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1007" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1007" s="16" t="s">
+      <c r="C1007" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1007" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1007" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1008" spans="1:5">
-      <c r="A1008" s="19" t="s">
+      <c r="A1008" s="14" t="s">
         <v>546</v>
       </c>
-      <c r="B1008" s="15" t="s">
+      <c r="B1008" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1008" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1008" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1008" s="16" t="s">
+      <c r="C1008" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1008" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1008" s="10" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="1009" spans="1:5">
-      <c r="A1009" s="19" t="s">
+      <c r="A1009" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B1009" s="15" t="s">
+      <c r="B1009" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1009" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1009" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1009" s="16" t="s">
+      <c r="C1009" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1009" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1009" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1010" spans="1:5">
-      <c r="A1010" s="19" t="s">
+      <c r="A1010" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B1010" s="15" t="s">
+      <c r="B1010" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1010" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1010" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1010" s="16" t="s">
+      <c r="C1010" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1010" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1010" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1011" spans="1:5">
-      <c r="A1011" s="19" t="s">
+      <c r="A1011" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B1011" s="15" t="s">
+      <c r="B1011" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1011" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1011" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1011" s="16" t="s">
+      <c r="C1011" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1011" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1011" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1012" spans="1:5">
-      <c r="A1012" s="19" t="s">
+      <c r="A1012" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B1012" s="15" t="s">
+      <c r="B1012" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1012" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1012" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1012" s="16" t="s">
+      <c r="C1012" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1012" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1012" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1013" spans="1:5">
-      <c r="A1013" s="14" t="s">
+      <c r="A1013" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B1013" s="15" t="s">
+      <c r="B1013" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1013" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1013" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1013" s="16" t="s">
+      <c r="C1013" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1013" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1013" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1014" spans="1:5">
-      <c r="A1014" s="14" t="s">
+      <c r="A1014" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B1014" s="15" t="s">
+      <c r="B1014" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1014" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1014" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1014" s="16" t="s">
+      <c r="C1014" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1014" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1014" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1015" spans="1:5">
-      <c r="A1015" s="14" t="s">
+      <c r="A1015" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B1015" s="15" t="s">
+      <c r="B1015" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1015" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1015" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1015" s="16" t="s">
+      <c r="C1015" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1015" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1015" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1016" spans="1:5">
-      <c r="A1016" s="14" t="s">
+      <c r="A1016" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B1016" s="15" t="s">
+      <c r="B1016" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1016" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1016" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1016" s="16" t="s">
+      <c r="C1016" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1016" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1016" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1017" spans="1:5">
-      <c r="A1017" s="14" t="s">
+      <c r="A1017" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B1017" s="15" t="s">
+      <c r="B1017" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1017" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1017" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1017" s="16" t="s">
+      <c r="C1017" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1017" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1017" s="10" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="1018" spans="1:5">
-      <c r="A1018" s="14" t="s">
+      <c r="A1018" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="B1018" s="15" t="s">
+      <c r="B1018" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1018" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1018" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1018" s="16" t="s">
+      <c r="C1018" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1018" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1018" s="10" t="s">
         <v>375</v>
       </c>
     </row>
@@ -19652,16 +19640,16 @@
       <c r="A1019" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="B1019" s="15" t="s">
+      <c r="B1019" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1019" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1019" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1019" s="16" t="s">
+      <c r="C1019" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1019" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1019" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19669,16 +19657,16 @@
       <c r="A1020" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="B1020" s="15" t="s">
+      <c r="B1020" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1020" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1020" s="15" t="s">
+      <c r="C1020" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1020" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E1020" s="16" t="s">
+      <c r="E1020" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19686,16 +19674,16 @@
       <c r="A1021" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="B1021" s="15" t="s">
+      <c r="B1021" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1021" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1021" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1021" s="16" t="s">
+      <c r="C1021" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1021" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1021" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19703,16 +19691,16 @@
       <c r="A1022" s="1" t="s">
         <v>550</v>
       </c>
-      <c r="B1022" s="15" t="s">
+      <c r="B1022" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1022" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1022" s="15" t="s">
+      <c r="C1022" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1022" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="E1022" s="16" t="s">
+      <c r="E1022" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19720,16 +19708,16 @@
       <c r="A1023" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B1023" s="15" t="s">
+      <c r="B1023" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1023" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1023" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1023" s="16" t="s">
+      <c r="C1023" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1023" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1023" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19737,16 +19725,16 @@
       <c r="A1024" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="B1024" s="15" t="s">
+      <c r="B1024" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C1024" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1024" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1024" s="16" t="s">
+      <c r="C1024" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1024" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1024" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19757,13 +19745,13 @@
       <c r="B1025" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1025" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1025" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1025" s="16" t="s">
+      <c r="C1025" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1025" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1025" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19774,13 +19762,13 @@
       <c r="B1026" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1026" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1026" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1026" s="16" t="s">
+      <c r="C1026" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1026" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1026" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19791,13 +19779,13 @@
       <c r="B1027" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1027" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1027" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1027" s="16" t="s">
+      <c r="C1027" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1027" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1027" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19808,13 +19796,13 @@
       <c r="B1028" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1028" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1028" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1028" s="16" t="s">
+      <c r="C1028" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1028" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1028" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19825,13 +19813,13 @@
       <c r="B1029" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1029" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1029" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1029" s="16" t="s">
+      <c r="C1029" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1029" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1029" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19842,13 +19830,13 @@
       <c r="B1030" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1030" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1030" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1030" s="16" t="s">
+      <c r="C1030" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1030" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1030" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19859,13 +19847,13 @@
       <c r="B1031" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1031" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1031" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1031" s="16" t="s">
+      <c r="C1031" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1031" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1031" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19876,13 +19864,13 @@
       <c r="B1032" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1032" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1032" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1032" s="16" t="s">
+      <c r="C1032" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1032" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1032" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19893,13 +19881,13 @@
       <c r="B1033" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1033" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1033" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1033" s="16" t="s">
+      <c r="C1033" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1033" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1033" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19910,13 +19898,13 @@
       <c r="B1034" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1034" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1034" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1034" s="16" t="s">
+      <c r="C1034" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1034" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1034" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19927,13 +19915,13 @@
       <c r="B1035" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1035" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1035" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1035" s="16" t="s">
+      <c r="C1035" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1035" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1035" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19944,13 +19932,13 @@
       <c r="B1036" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1036" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1036" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1036" s="16" t="s">
+      <c r="C1036" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1036" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1036" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19961,13 +19949,13 @@
       <c r="B1037" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1037" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1037" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1037" s="16" t="s">
+      <c r="C1037" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1037" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1037" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19978,13 +19966,13 @@
       <c r="B1038" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1038" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1038" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1038" s="16" t="s">
+      <c r="C1038" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1038" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1038" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -19995,13 +19983,13 @@
       <c r="B1039" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1039" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1039" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1039" s="16" t="s">
+      <c r="C1039" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1039" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1039" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20012,13 +20000,13 @@
       <c r="B1040" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1040" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1040" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1040" s="16" t="s">
+      <c r="C1040" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1040" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1040" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20029,13 +20017,13 @@
       <c r="B1041" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1041" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1041" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1041" s="16" t="s">
+      <c r="C1041" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1041" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1041" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20046,13 +20034,13 @@
       <c r="B1042" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1042" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1042" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1042" s="16" t="s">
+      <c r="C1042" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1042" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1042" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20063,13 +20051,13 @@
       <c r="B1043" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="C1043" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1043" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1043" s="16" t="s">
+      <c r="C1043" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1043" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1043" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20080,13 +20068,13 @@
       <c r="B1044" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1044" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1044" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1044" s="16" t="s">
+      <c r="C1044" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1044" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1044" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20097,13 +20085,13 @@
       <c r="B1045" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1045" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1045" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1045" s="16" t="s">
+      <c r="C1045" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1045" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1045" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20114,13 +20102,13 @@
       <c r="B1046" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1046" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1046" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1046" s="16" t="s">
+      <c r="C1046" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1046" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1046" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20131,13 +20119,13 @@
       <c r="B1047" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1047" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1047" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1047" s="16" t="s">
+      <c r="C1047" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1047" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1047" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20148,13 +20136,13 @@
       <c r="B1048" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1048" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1048" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1048" s="16" t="s">
+      <c r="C1048" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1048" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1048" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20165,13 +20153,13 @@
       <c r="B1049" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1049" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1049" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1049" s="16" t="s">
+      <c r="C1049" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1049" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1049" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20182,13 +20170,13 @@
       <c r="B1050" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1050" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1050" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1050" s="16" t="s">
+      <c r="C1050" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1050" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1050" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20199,13 +20187,13 @@
       <c r="B1051" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1051" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1051" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1051" s="16" t="s">
+      <c r="C1051" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1051" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1051" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20216,13 +20204,13 @@
       <c r="B1052" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1052" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1052" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1052" s="16" t="s">
+      <c r="C1052" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1052" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1052" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20233,13 +20221,13 @@
       <c r="B1053" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1053" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1053" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1053" s="16" t="s">
+      <c r="C1053" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1053" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1053" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20250,13 +20238,13 @@
       <c r="B1054" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1054" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1054" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1054" s="16" t="s">
+      <c r="C1054" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1054" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1054" s="10" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20267,13 +20255,13 @@
       <c r="B1055" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C1055" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1055" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1055" s="20" t="s">
+      <c r="C1055" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1055" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1055" s="15" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20290,7 +20278,7 @@
       <c r="D1056" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1056" s="20" t="s">
+      <c r="E1056" s="15" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20307,7 +20295,7 @@
       <c r="D1057" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1057" s="20" t="s">
+      <c r="E1057" s="15" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20318,13 +20306,13 @@
       <c r="B1058" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C1058" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1058" s="21" t="s">
+      <c r="C1058" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1058" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E1058" s="20" t="s">
+      <c r="E1058" s="15" t="s">
         <v>365</v>
       </c>
     </row>
@@ -20342,6 +20330,23 @@
         <v>42</v>
       </c>
       <c r="E1059" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:5">
+      <c r="A1060" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1060" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1060" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1060" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1060" s="2" t="s">
         <v>365</v>
       </c>
     </row>

</xml_diff>